<commit_message>
Update manual test, templates, and metadata
Replace two resource templates (protocol_schema_iphra.xlsx and reach_tor_iphra_template.docx) and adjust the manual protocol workflow test. In tests/manual/test_manual_protocol_workflow.R: replace head(...$revised_survey) with View(...), remove several metadata assignments (pop_host, pop_idphost, popsize_known_geographic_unit, geographic_coverage) and the protocol$update_metadata(...) call, keep popsize_known_strata_unit, shorten secondary_data entry 101 to "ACLED", and add/adjust a few commented lines and spacing. These changes tidy up the test script and update bundled templates.
</commit_message>
<xml_diff>
--- a/inst/resources/protocol_schema_iphra.xlsx
+++ b/inst/resources/protocol_schema_iphra.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R Projects\SaeedR1987\public_health_resources\inst\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saeed.rahman\Desktop\public_health_resources\inst\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D02E6903-5556-438A-ACEC-D6865094572A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC0529E9-B895-4AE4-91B6-51997D41A55A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2175" yWindow="3000" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="schema" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="228">
   <si>
     <t>tag_name</t>
   </si>
@@ -492,13 +492,240 @@
   </si>
   <si>
     <t xml:space="preserve">In cases where no MUAC or mortality data is being collected, the sample size can be estimated based on other household level indicators such as FSL and WASH. The below table summarizes the sampling assumptions for each strata. </t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>character</t>
+  </si>
+  <si>
+    <t>handling</t>
+  </si>
+  <si>
+    <t>@tor_title</t>
+  </si>
+  <si>
+    <t>Research Terms of Reference</t>
+  </si>
+  <si>
+    <t>@research_cycle_title</t>
+  </si>
+  <si>
+    <t>@research_cycle_id</t>
+  </si>
+  <si>
+    <t>Integrated Public Health Rapid Assessment (IPHRA)</t>
+  </si>
+  <si>
+    <t>Research Cycle ID</t>
+  </si>
+  <si>
+    <t>replace</t>
+  </si>
+  <si>
+    <t>calculate</t>
+  </si>
+  <si>
+    <t>checkbox_replace</t>
+  </si>
+  <si>
+    <t>@header_exec_summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Executive Summary </t>
+  </si>
+  <si>
+    <t>@header_country</t>
+  </si>
+  <si>
+    <t>Country of intervention</t>
+  </si>
+  <si>
+    <t>@header_type_emergency</t>
+  </si>
+  <si>
+    <t>Type of Emergency</t>
+  </si>
+  <si>
+    <t>Type of Crisis</t>
+  </si>
+  <si>
+    <t>@header_type_crisis</t>
+  </si>
+  <si>
+    <t>@header_crisis_natural_disaster</t>
+  </si>
+  <si>
+    <t>@header_crisis_conflict</t>
+  </si>
+  <si>
+    <t>@header_crisis_other</t>
+  </si>
+  <si>
+    <t>@header_crisis_sudden_onset</t>
+  </si>
+  <si>
+    <t>@header_crisis_slow_onset</t>
+  </si>
+  <si>
+    <t>@header_crisis_protracted</t>
+  </si>
+  <si>
+    <t>Natural disaster</t>
+  </si>
+  <si>
+    <t>Conflict</t>
+  </si>
+  <si>
+    <t>Protracted</t>
+  </si>
+  <si>
+    <t>Other (Specify)</t>
+  </si>
+  <si>
+    <t>Sudden Onset</t>
+  </si>
+  <si>
+    <t>Slow Onset</t>
+  </si>
+  <si>
+    <t>@header_mandating_agency</t>
+  </si>
+  <si>
+    <t>Mandating Body/ Agency</t>
+  </si>
+  <si>
+    <t>IMPACT Project Code</t>
+  </si>
+  <si>
+    <t>@header_impact_project_code</t>
+  </si>
+  <si>
+    <t>@header_overall_timeframe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Overall Research Timeframe </t>
+  </si>
+  <si>
+    <t>@header_research_timeframe</t>
+  </si>
+  <si>
+    <t>Research Timeframe</t>
+  </si>
+  <si>
+    <t>input</t>
+  </si>
+  <si>
+    <t>@header_pilot_date</t>
+  </si>
+  <si>
+    <t>Pilot/ training:</t>
+  </si>
+  <si>
+    <t>@header_data_start_date</t>
+  </si>
+  <si>
+    <t>@header_data_end_date</t>
+  </si>
+  <si>
+    <t>@header_analysis_date</t>
+  </si>
+  <si>
+    <t>@header_data_validation_date</t>
+  </si>
+  <si>
+    <t>@header_prelim_presentation_date</t>
+  </si>
+  <si>
+    <t>@header_output_validation_date</t>
+  </si>
+  <si>
+    <t>@header_output_published_date</t>
+  </si>
+  <si>
+    <t>@header_final_presentation_date</t>
+  </si>
+  <si>
+    <t>@crisis_other</t>
+  </si>
+  <si>
+    <t>@crisis_conflict</t>
+  </si>
+  <si>
+    <t>@crisis_natural_disaster</t>
+  </si>
+  <si>
+    <t>@crisis_sudden_onset</t>
+  </si>
+  <si>
+    <t>@crisis_slow_onset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data collected: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Start collect data: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data analysed: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data sent for validation: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preliminary presentation: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outputs sent for validation: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outputs published: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Final presentation: </t>
+  </si>
+  <si>
+    <t>@header_humanitarian_milestone</t>
+  </si>
+  <si>
+    <t>@header_milestone</t>
+  </si>
+  <si>
+    <t>@header_deadline</t>
+  </si>
+  <si>
+    <t>Deadline (can be tentative)</t>
+  </si>
+  <si>
+    <t>Milestone</t>
+  </si>
+  <si>
+    <t>Humanitarian milestones
+Specify what will the assessment inform and when 
+e.g. The shelter cluster will use this data to draft its Revised Flash Appeal;</t>
+  </si>
+  <si>
+    <t>@header_milestone_donor</t>
+  </si>
+  <si>
+    <t>@header_milestone_intercluster</t>
+  </si>
+  <si>
+    <t>@header_milestone_cluster</t>
+  </si>
+  <si>
+    <t>@header_milestone_ngo_platform</t>
+  </si>
+  <si>
+    <t>@header_milestone_other</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -510,6 +737,47 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFEE5859"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -532,10 +800,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -838,938 +1125,1565 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B139"/>
+  <dimension ref="A1:D188"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="56.5703125" customWidth="1"/>
-    <col min="2" max="2" width="80" customWidth="1"/>
+    <col min="1" max="1" width="33.85546875" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" customWidth="1"/>
+    <col min="4" max="4" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="C2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="C3" t="s">
+        <v>154</v>
+      </c>
+      <c r="D3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="C4" t="s">
+        <v>154</v>
+      </c>
+      <c r="D4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="9" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B6" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="C6" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B7" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="C7" t="s">
+        <v>154</v>
+      </c>
+      <c r="D7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="8" spans="1:4" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="C8" t="s">
+        <v>154</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="D13" s="12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="D15" s="12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="D17" s="12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="D19" s="12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="D21" s="12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A22" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="D23" s="12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B25" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A26" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="B27" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A28" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="B29" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A31" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>14</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A33" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D33" s="10" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>15</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A35" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D35" s="10" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>16</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A37" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D37" s="10" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>17</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A39" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>18</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A41" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D41" s="10" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>19</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A43" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D43" s="10" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>20</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D45" s="10" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>21</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D47" s="10" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>22</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D49" s="13" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D50" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B52" s="5" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B53" s="5" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B54" s="5" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B55" s="5" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="2"/>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="2"/>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
         <v>11</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B61" t="s">
+        <v>162</v>
+      </c>
+      <c r="D61" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
         <v>23</v>
       </c>
-      <c r="B21" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="B70" t="s">
+        <v>164</v>
+      </c>
+      <c r="D70" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
         <v>25</v>
       </c>
-      <c r="B22" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="B71" t="s">
+        <v>164</v>
+      </c>
+      <c r="D71" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
         <v>26</v>
       </c>
-      <c r="B23" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="B72" t="s">
+        <v>164</v>
+      </c>
+      <c r="D72" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
         <v>27</v>
       </c>
-      <c r="B24" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+      <c r="B73" t="s">
+        <v>164</v>
+      </c>
+      <c r="D73" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
         <v>28</v>
       </c>
-      <c r="B25" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+      <c r="B74" t="s">
+        <v>164</v>
+      </c>
+      <c r="D74" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
         <v>29</v>
       </c>
-      <c r="B26" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+      <c r="B75" t="s">
+        <v>164</v>
+      </c>
+      <c r="D75" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
         <v>30</v>
       </c>
-      <c r="B27" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+      <c r="B76" t="s">
+        <v>164</v>
+      </c>
+      <c r="D76" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
         <v>31</v>
       </c>
-      <c r="B28" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+      <c r="B77" t="s">
+        <v>164</v>
+      </c>
+      <c r="D77" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
         <v>32</v>
       </c>
-      <c r="B29" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+      <c r="B78" t="s">
+        <v>164</v>
+      </c>
+      <c r="D78" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
         <v>33</v>
       </c>
-      <c r="B30" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="B79" t="s">
+        <v>164</v>
+      </c>
+      <c r="D79" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
         <v>34</v>
       </c>
-      <c r="B31" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="B80" t="s">
+        <v>164</v>
+      </c>
+      <c r="D80" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
         <v>35</v>
       </c>
-      <c r="B32" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+      <c r="B81" t="s">
+        <v>164</v>
+      </c>
+      <c r="D81" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
         <v>36</v>
       </c>
-      <c r="B33" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+      <c r="B82" t="s">
+        <v>164</v>
+      </c>
+      <c r="D82" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
         <v>37</v>
       </c>
-      <c r="B34" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+      <c r="B83" t="s">
+        <v>164</v>
+      </c>
+      <c r="D83" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
         <v>38</v>
       </c>
-      <c r="B35" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+      <c r="B84" t="s">
+        <v>164</v>
+      </c>
+      <c r="D84" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
         <v>39</v>
       </c>
-      <c r="B36" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+      <c r="B85" t="s">
+        <v>164</v>
+      </c>
+      <c r="D85" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
         <v>40</v>
       </c>
-      <c r="B37" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+      <c r="B86" t="s">
+        <v>164</v>
+      </c>
+      <c r="D86" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
         <v>41</v>
       </c>
-      <c r="B38" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+      <c r="B87" t="s">
+        <v>164</v>
+      </c>
+      <c r="D87" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
         <v>42</v>
       </c>
-      <c r="B39" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+      <c r="B88" t="s">
+        <v>164</v>
+      </c>
+      <c r="D88" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
         <v>43</v>
       </c>
-      <c r="B40" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+      <c r="B89" t="s">
+        <v>164</v>
+      </c>
+      <c r="D89" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
         <v>44</v>
       </c>
-      <c r="B41" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+      <c r="B90" t="s">
+        <v>164</v>
+      </c>
+      <c r="D90" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
         <v>45</v>
       </c>
-      <c r="B42" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+      <c r="B91" t="s">
+        <v>164</v>
+      </c>
+      <c r="D91" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
         <v>46</v>
       </c>
-      <c r="B43" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+      <c r="B92" t="s">
+        <v>164</v>
+      </c>
+      <c r="D92" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
         <v>47</v>
       </c>
-      <c r="B44" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+      <c r="B93" t="s">
+        <v>164</v>
+      </c>
+      <c r="D93" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
         <v>48</v>
       </c>
-      <c r="B45" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+      <c r="B94" t="s">
+        <v>164</v>
+      </c>
+      <c r="D94" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
         <v>49</v>
       </c>
-      <c r="B46" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+      <c r="B95" t="s">
+        <v>164</v>
+      </c>
+      <c r="D95" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
         <v>50</v>
       </c>
-      <c r="B47" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
+      <c r="B96" t="s">
+        <v>164</v>
+      </c>
+      <c r="D96" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
         <v>51</v>
       </c>
-      <c r="B48" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
+      <c r="B97" t="s">
+        <v>164</v>
+      </c>
+      <c r="D97" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
         <v>52</v>
       </c>
-      <c r="B49" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+      <c r="B98" t="s">
+        <v>164</v>
+      </c>
+      <c r="D98" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
         <v>53</v>
       </c>
-      <c r="B50" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
+      <c r="B99" t="s">
+        <v>164</v>
+      </c>
+      <c r="D99" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
         <v>54</v>
       </c>
-      <c r="B51" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
+      <c r="B100" t="s">
+        <v>164</v>
+      </c>
+      <c r="D100" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
         <v>55</v>
       </c>
-      <c r="B52" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
+      <c r="B101" t="s">
+        <v>164</v>
+      </c>
+      <c r="D101" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
         <v>57</v>
       </c>
-      <c r="B54" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+      <c r="D103" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
         <v>58</v>
       </c>
-      <c r="B55" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
+      <c r="D104" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
         <v>59</v>
       </c>
-      <c r="B56" t="s">
+      <c r="D105" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
         <v>61</v>
       </c>
-      <c r="B57" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
+      <c r="D106" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
         <v>62</v>
       </c>
-      <c r="B58" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
+      <c r="D107" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
         <v>74</v>
       </c>
-      <c r="B70" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
+      <c r="D119" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
         <v>75</v>
       </c>
-      <c r="B71" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
+      <c r="D120" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
         <v>76</v>
       </c>
-      <c r="B72" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+      <c r="D121" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
         <v>77</v>
       </c>
-      <c r="B73" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
+      <c r="D122" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
         <v>78</v>
       </c>
-      <c r="B74" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
+      <c r="D123" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
         <v>79</v>
       </c>
-      <c r="B75" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
+      <c r="D124" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
         <v>80</v>
       </c>
-      <c r="B76" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
+      <c r="D125" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
         <v>81</v>
       </c>
-      <c r="B77" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
+      <c r="D126" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
         <v>82</v>
       </c>
-      <c r="B78" t="s">
+      <c r="D127" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
         <v>84</v>
       </c>
-      <c r="B79" t="s">
+      <c r="D128" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
         <v>98</v>
       </c>
-      <c r="B93" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
+      <c r="D142" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
         <v>99</v>
       </c>
-      <c r="B94" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
+      <c r="D143" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
         <v>100</v>
       </c>
-      <c r="B95" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
+      <c r="D144" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
         <v>101</v>
       </c>
-      <c r="B96" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
+      <c r="D145" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
         <v>102</v>
       </c>
-      <c r="B97" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
+      <c r="D146" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
         <v>103</v>
       </c>
-      <c r="B98" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
+      <c r="D147" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
         <v>104</v>
       </c>
-      <c r="B99" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
+      <c r="D148" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
         <v>105</v>
       </c>
-      <c r="B100" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
+      <c r="D149" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
         <v>106</v>
       </c>
-      <c r="B101" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
+      <c r="D150" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
         <v>107</v>
       </c>
-      <c r="B102" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
+      <c r="D151" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
         <v>108</v>
       </c>
-      <c r="B103" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
+      <c r="D152" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
         <v>109</v>
       </c>
-      <c r="B104" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
+      <c r="D153" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
         <v>110</v>
       </c>
-      <c r="B105" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
+      <c r="D154" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
         <v>111</v>
       </c>
-      <c r="B106" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A107" t="s">
+      <c r="D155" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
         <v>112</v>
       </c>
-      <c r="B107" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
+      <c r="D156" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
         <v>113</v>
       </c>
-      <c r="B108" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
+      <c r="D157" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
         <v>114</v>
       </c>
-      <c r="B109" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
+      <c r="D158" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A114" t="s">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A120" t="s">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
         <v>125</v>
       </c>
-      <c r="B120" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
+      <c r="D169" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
         <v>126</v>
       </c>
-      <c r="B121" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
+      <c r="D170" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A124" t="s">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A127" s="2" t="s">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A176" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B127" t="s">
+      <c r="B176" s="2"/>
+      <c r="C176" s="2"/>
+      <c r="D176" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A128" s="2" t="s">
+    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A177" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B128" t="s">
+      <c r="B177" s="2"/>
+      <c r="C177" s="2"/>
+      <c r="D177" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A129" s="2" t="s">
+    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A178" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B129" t="s">
+      <c r="B178" s="2"/>
+      <c r="C178" s="2"/>
+      <c r="D178" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A130" s="2" t="s">
+    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A179" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="B130" t="s">
+      <c r="B179" s="2"/>
+      <c r="C179" s="2"/>
+      <c r="D179" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A131" s="2" t="s">
+    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A180" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="B131" t="s">
+      <c r="B180" s="2"/>
+      <c r="C180" s="2"/>
+      <c r="D180" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A132" s="2" t="s">
+    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A181" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="B132" t="s">
+      <c r="B181" s="2"/>
+      <c r="C181" s="2"/>
+      <c r="D181" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A133" s="2" t="s">
+    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A182" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="B133" t="s">
+      <c r="B182" s="2"/>
+      <c r="C182" s="2"/>
+      <c r="D182" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A134" s="2" t="s">
+    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A183" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="B134" t="s">
+      <c r="B183" s="2"/>
+      <c r="C183" s="2"/>
+      <c r="D183" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A135" s="2" t="s">
+    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A184" s="2" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A136" s="2" t="s">
+      <c r="B184" s="2"/>
+      <c r="C184" s="2"/>
+    </row>
+    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A185" s="2" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A137" s="2" t="s">
+      <c r="B185" s="2"/>
+      <c r="C185" s="2"/>
+    </row>
+    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A186" s="2" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A138" s="2" t="s">
+      <c r="B186" s="2"/>
+      <c r="C186" s="2"/>
+    </row>
+    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A187" s="2" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A139" s="2" t="s">
+      <c r="B187" s="2"/>
+      <c r="C187" s="2"/>
+    </row>
+    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A188" s="2" t="s">
         <v>151</v>
       </c>
+      <c r="B188" s="2"/>
+      <c r="C188" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update IPHRA protocol schema and template
Replace inst/resources/protocol_schema_iphra.xlsx and inst/resources/reach_tor_iphra_template.docx with updated versions. These changes update the IPHRA protocol schema spreadsheet and the REACH TOR template document (content/format revisions); no source code was modified.
</commit_message>
<xml_diff>
--- a/inst/resources/protocol_schema_iphra.xlsx
+++ b/inst/resources/protocol_schema_iphra.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R Projects\SaeedR1987\public_health_resources\inst\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16AFBCCB-0010-4767-8C7C-316D7B9CF0B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7977D509-C76A-44CF-A89E-AFB9B54262F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14595" yWindow="0" windowWidth="14685" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="schema" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1119" uniqueCount="673">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1147" uniqueCount="693">
   <si>
     <t>tag_name</t>
   </si>
@@ -2161,9 +2161,6 @@
     <t>kii_wash_provider</t>
   </si>
   <si>
-    <t xml:space="preserve">Service provider key informant interviews will be purposefully selected based on staff available for interview. These staff should be individuals with direct knowledge or involvement in service provision for the affected population. @text_kii_health_facility . @text_kii_nutrition_facility . @text_kii_fsl_provider . @text_kii_wash_provider . One interview will be conducted with staff from each health facility or service provider NGO in the assessment area. Eligible staff are preferably program or facility managers with an understanding of the service delivery challenges but may also be senior officers, health or nutrition practitioners if needed. </t>
-  </si>
-  <si>
     <t>nutrition facilities,</t>
   </si>
   <si>
@@ -2177,6 +2174,69 @@
   </si>
   <si>
     <t>@text_methodology_obs_community</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service provider key informant interviews will be purposefully selected based on staff available for interview. These staff should be individuals with direct knowledge or involvement in service provision for the affected population. This includes interviews with staff from: @text_kii_health_facility , @text_kii_nutrition_facility , @text_kii_fsl_provider , @text_kii_wash_provider . One interview will be conducted with staff from each health facility or service provider NGO in the assessment area. Eligible staff are preferably program or facility managers with an understanding of the service delivery challenges but may also be senior officers, health or nutrition practitioners if needed. </t>
+  </si>
+  <si>
+    <t>@text_methodology_obs_service_providers</t>
+  </si>
+  <si>
+    <t>obs_community</t>
+  </si>
+  <si>
+    <t>obs_service_providers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Community observation checklists will be implemented in each assessed site to triangulate observable facts against household and key informant reporting. Observations will be made by making a transect walk through the community focusing on environmental conditions, damage, and community norms. </t>
+  </si>
+  <si>
+    <t>@text_obs_water_point</t>
+  </si>
+  <si>
+    <t>@text_obs_latrines</t>
+  </si>
+  <si>
+    <t>obs_water_point</t>
+  </si>
+  <si>
+    <t>obs_latrines</t>
+  </si>
+  <si>
+    <t>obs_health_facility</t>
+  </si>
+  <si>
+    <t>obs_crops_livestock</t>
+  </si>
+  <si>
+    <t>@text_obs_health_facility</t>
+  </si>
+  <si>
+    <t>@text_obs_crops_livestock</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Specialized observation tools will be implemented at @text_obs_water_point , @text_obs_latrines , @text_obs_health_facility to evaluate basic infrastructure and functionality. @text_obs_crops_livestock . </t>
+  </si>
+  <si>
+    <t>water points</t>
+  </si>
+  <si>
+    <t>latrines</t>
+  </si>
+  <si>
+    <t>health facilities</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An observation tool will be used to assess the condition of crops and/or livestock in the community using a transect walk through purposively selected locations. </t>
+  </si>
+  <si>
+    <t>@header_population_of_interest</t>
+  </si>
+  <si>
+    <t>Population of interest</t>
+  </si>
+  <si>
+    <t>@total_population_size</t>
   </si>
 </sst>
 </file>
@@ -2733,7 +2793,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D425"/>
+  <dimension ref="A1:D437"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="53.140625" customWidth="1"/>
@@ -6524,7 +6584,7 @@
       <c r="D377" s="27"/>
     </row>
     <row r="378" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A378" s="27" t="s">
+      <c r="A378" s="36" t="s">
         <v>654</v>
       </c>
       <c r="B378" t="s">
@@ -6548,7 +6608,7 @@
         <v>662</v>
       </c>
       <c r="D379" s="27" t="s">
-        <v>667</v>
+        <v>672</v>
       </c>
     </row>
     <row r="380" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -6562,7 +6622,7 @@
         <v>663</v>
       </c>
       <c r="D380" s="27" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="381" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -6576,7 +6636,7 @@
         <v>664</v>
       </c>
       <c r="D381" s="27" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="382" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -6590,7 +6650,7 @@
         <v>665</v>
       </c>
       <c r="D382" s="27" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="383" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -6604,417 +6664,536 @@
         <v>666</v>
       </c>
       <c r="D383" s="27" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="384" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A384" s="37" t="s">
         <v>671</v>
       </c>
-    </row>
-    <row r="384" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A384" s="2"/>
-      <c r="C384" s="2"/>
-      <c r="D384" s="27"/>
+      <c r="B384" t="s">
+        <v>499</v>
+      </c>
+      <c r="C384" s="2" t="s">
+        <v>674</v>
+      </c>
+      <c r="D384" s="27" t="s">
+        <v>676</v>
+      </c>
     </row>
     <row r="385" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A385" s="37" t="s">
-        <v>672</v>
-      </c>
-      <c r="C385" s="2"/>
-      <c r="D385" s="27"/>
+        <v>673</v>
+      </c>
+      <c r="B385" t="s">
+        <v>499</v>
+      </c>
+      <c r="C385" s="2" t="s">
+        <v>675</v>
+      </c>
+      <c r="D385" s="27" t="s">
+        <v>685</v>
+      </c>
     </row>
     <row r="386" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A386" s="2"/>
-      <c r="C386" s="2"/>
-      <c r="D386" s="27"/>
+      <c r="A386" s="36" t="s">
+        <v>677</v>
+      </c>
+      <c r="B386" t="s">
+        <v>499</v>
+      </c>
+      <c r="C386" s="2" t="s">
+        <v>679</v>
+      </c>
+      <c r="D386" s="27" t="s">
+        <v>686</v>
+      </c>
     </row>
     <row r="387" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A387" s="2"/>
-      <c r="C387" s="2"/>
-      <c r="D387" s="27"/>
+      <c r="A387" s="36" t="s">
+        <v>678</v>
+      </c>
+      <c r="B387" t="s">
+        <v>499</v>
+      </c>
+      <c r="C387" s="2" t="s">
+        <v>680</v>
+      </c>
+      <c r="D387" s="27" t="s">
+        <v>687</v>
+      </c>
     </row>
     <row r="388" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A388" s="2"/>
-      <c r="C388" s="2"/>
-      <c r="D388" s="27"/>
+      <c r="A388" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="B388" t="s">
+        <v>499</v>
+      </c>
+      <c r="C388" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="D388" s="27" t="s">
+        <v>688</v>
+      </c>
     </row>
     <row r="389" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A389" s="2"/>
-      <c r="C389" s="2"/>
-      <c r="D389" s="27"/>
-    </row>
-    <row r="390" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A390" s="2"/>
-      <c r="C390" s="2"/>
-      <c r="D390" s="27"/>
-    </row>
-    <row r="391" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A391" s="2"/>
+      <c r="A389" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="B389" t="s">
+        <v>499</v>
+      </c>
+      <c r="C389" s="2" t="s">
+        <v>682</v>
+      </c>
+      <c r="D389" s="27" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="390" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A390" t="s">
+        <v>113</v>
+      </c>
+      <c r="B390" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="391" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A391" s="2" t="s">
+        <v>690</v>
+      </c>
+      <c r="B391" t="s">
+        <v>140</v>
+      </c>
       <c r="C391" s="2"/>
-      <c r="D391" s="27"/>
+      <c r="D391" s="26" t="s">
+        <v>691</v>
+      </c>
     </row>
     <row r="392" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A392" s="2"/>
+      <c r="A392" s="2" t="s">
+        <v>692</v>
+      </c>
+      <c r="B392" t="s">
+        <v>141</v>
+      </c>
       <c r="C392" s="2"/>
       <c r="D392" s="27"/>
     </row>
-    <row r="393" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A393" t="s">
-        <v>113</v>
-      </c>
-      <c r="B393" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="394" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A394" s="2" t="s">
+    <row r="393" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A393" s="2"/>
+      <c r="C393" s="2"/>
+      <c r="D393" s="27"/>
+    </row>
+    <row r="394" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A394" s="2"/>
+      <c r="C394" s="2"/>
+      <c r="D394" s="27"/>
+    </row>
+    <row r="395" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A395" s="2"/>
+      <c r="C395" s="2"/>
+      <c r="D395" s="27"/>
+    </row>
+    <row r="396" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A396" s="2"/>
+      <c r="C396" s="2"/>
+      <c r="D396" s="27"/>
+    </row>
+    <row r="397" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A397" s="2"/>
+      <c r="C397" s="2"/>
+      <c r="D397" s="27"/>
+    </row>
+    <row r="398" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A398" s="2"/>
+      <c r="C398" s="2"/>
+      <c r="D398" s="27"/>
+    </row>
+    <row r="399" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A399" s="2"/>
+      <c r="C399" s="2"/>
+      <c r="D399" s="27"/>
+    </row>
+    <row r="400" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A400" s="2"/>
+      <c r="C400" s="2"/>
+      <c r="D400" s="27"/>
+    </row>
+    <row r="401" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A401" s="2"/>
+      <c r="C401" s="2"/>
+      <c r="D401" s="27"/>
+    </row>
+    <row r="402" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A402" s="2"/>
+      <c r="C402" s="2"/>
+      <c r="D402" s="27"/>
+    </row>
+    <row r="403" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A403" s="2"/>
+      <c r="C403" s="2"/>
+      <c r="D403" s="27"/>
+    </row>
+    <row r="404" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A404" s="2"/>
+      <c r="C404" s="2"/>
+      <c r="D404" s="27"/>
+    </row>
+    <row r="406" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A406" s="2" t="s">
         <v>549</v>
       </c>
-      <c r="B394" t="s">
-        <v>140</v>
-      </c>
-      <c r="D394" s="26" t="s">
+      <c r="B406" t="s">
+        <v>140</v>
+      </c>
+      <c r="D406" s="26" t="s">
         <v>551</v>
       </c>
     </row>
-    <row r="395" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A395" s="2" t="s">
+    <row r="407" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A407" s="2" t="s">
         <v>550</v>
       </c>
-      <c r="B395" t="s">
-        <v>140</v>
-      </c>
-      <c r="D395" s="27" t="s">
+      <c r="B407" t="s">
+        <v>140</v>
+      </c>
+      <c r="D407" s="27" t="s">
         <v>552</v>
       </c>
     </row>
-    <row r="396" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A396" t="s">
+    <row r="408" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A408" t="s">
         <v>114</v>
       </c>
-      <c r="B396" t="s">
+      <c r="B408" t="s">
         <v>511</v>
-      </c>
-    </row>
-    <row r="397" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A397" s="2" t="s">
-        <v>553</v>
-      </c>
-      <c r="B397" t="s">
-        <v>140</v>
-      </c>
-      <c r="D397" t="s">
-        <v>554</v>
-      </c>
-    </row>
-    <row r="398" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A398" t="s">
-        <v>115</v>
-      </c>
-      <c r="B398" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="399" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A399" s="2" t="s">
-        <v>547</v>
-      </c>
-      <c r="B399" t="s">
-        <v>140</v>
-      </c>
-      <c r="D399" s="33" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="400" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A400" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="B400" t="s">
-        <v>499</v>
-      </c>
-      <c r="C400" s="2" t="s">
-        <v>513</v>
-      </c>
-      <c r="D400" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="401" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A401" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="B401" t="s">
-        <v>499</v>
-      </c>
-      <c r="C401" s="2" t="s">
-        <v>519</v>
-      </c>
-      <c r="D401" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="402" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A402" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="B402" t="s">
-        <v>499</v>
-      </c>
-      <c r="C402" s="2" t="s">
-        <v>514</v>
-      </c>
-      <c r="D402" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="403" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A403" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B403" t="s">
-        <v>499</v>
-      </c>
-      <c r="C403" s="2" t="s">
-        <v>515</v>
-      </c>
-      <c r="D403" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="404" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A404" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B404" t="s">
-        <v>499</v>
-      </c>
-      <c r="C404" s="2" t="s">
-        <v>516</v>
-      </c>
-      <c r="D404" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="405" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A405" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="B405" t="s">
-        <v>499</v>
-      </c>
-      <c r="C405" s="2" t="s">
-        <v>517</v>
-      </c>
-      <c r="D405" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="406" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A406" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="B406" t="s">
-        <v>499</v>
-      </c>
-      <c r="C406" s="2" t="s">
-        <v>518</v>
-      </c>
-      <c r="D406" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="407" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A407" s="2" t="s">
-        <v>543</v>
-      </c>
-      <c r="B407" t="s">
-        <v>140</v>
-      </c>
-      <c r="C407" s="2"/>
-      <c r="D407" s="26" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="408" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A408" s="2" t="s">
-        <v>545</v>
-      </c>
-      <c r="B408" t="s">
-        <v>140</v>
-      </c>
-      <c r="C408" s="2"/>
-      <c r="D408" s="10" t="s">
-        <v>546</v>
       </c>
     </row>
     <row r="409" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A409" s="2" t="s">
-        <v>522</v>
+        <v>553</v>
       </c>
       <c r="B409" t="s">
-        <v>499</v>
-      </c>
-      <c r="C409" s="2" t="s">
-        <v>523</v>
+        <v>140</v>
       </c>
       <c r="D409" t="s">
-        <v>526</v>
+        <v>554</v>
       </c>
     </row>
     <row r="410" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A410" s="2" t="s">
-        <v>530</v>
+      <c r="A410" t="s">
+        <v>115</v>
       </c>
       <c r="B410" t="s">
-        <v>499</v>
-      </c>
-      <c r="C410" s="2" t="s">
-        <v>524</v>
-      </c>
-      <c r="D410" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="411" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A411" s="30" t="s">
-        <v>537</v>
+        <v>510</v>
+      </c>
+    </row>
+    <row r="411" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A411" s="2" t="s">
+        <v>547</v>
       </c>
       <c r="B411" t="s">
-        <v>499</v>
-      </c>
-      <c r="C411" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="D411" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="412" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A412" s="30" t="s">
-        <v>538</v>
+        <v>140</v>
+      </c>
+      <c r="D411" s="33" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="412" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A412" s="2" t="s">
+        <v>128</v>
       </c>
       <c r="B412" t="s">
         <v>499</v>
       </c>
       <c r="C412" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="D412" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="413" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A413" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B413" t="s">
+        <v>499</v>
+      </c>
+      <c r="C413" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="D413" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="414" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A414" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B414" t="s">
+        <v>499</v>
+      </c>
+      <c r="C414" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="D414" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="415" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A415" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B415" t="s">
+        <v>499</v>
+      </c>
+      <c r="C415" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="D415" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="416" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A416" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B416" t="s">
+        <v>499</v>
+      </c>
+      <c r="C416" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="D416" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="417" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A417" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B417" t="s">
+        <v>499</v>
+      </c>
+      <c r="C417" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="D417" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="418" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A418" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B418" t="s">
+        <v>499</v>
+      </c>
+      <c r="C418" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="D418" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="419" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A419" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="B419" t="s">
+        <v>140</v>
+      </c>
+      <c r="C419" s="2"/>
+      <c r="D419" s="26" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="420" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A420" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="B420" t="s">
+        <v>140</v>
+      </c>
+      <c r="C420" s="2"/>
+      <c r="D420" s="10" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="421" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A421" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="B421" t="s">
+        <v>499</v>
+      </c>
+      <c r="C421" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="D421" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="422" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A422" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="B422" t="s">
+        <v>499</v>
+      </c>
+      <c r="C422" s="2" t="s">
+        <v>524</v>
+      </c>
+      <c r="D422" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="423" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A423" s="30" t="s">
+        <v>537</v>
+      </c>
+      <c r="B423" t="s">
+        <v>499</v>
+      </c>
+      <c r="C423" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="D423" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="424" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A424" s="30" t="s">
+        <v>538</v>
+      </c>
+      <c r="B424" t="s">
+        <v>499</v>
+      </c>
+      <c r="C424" s="2" t="s">
         <v>531</v>
       </c>
-      <c r="D412" t="s">
+      <c r="D424" t="s">
         <v>541</v>
       </c>
     </row>
-    <row r="413" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A413" s="28" t="s">
+    <row r="425" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A425" s="28" t="s">
         <v>520</v>
       </c>
-      <c r="B413" s="28" t="s">
+      <c r="B425" s="28" t="s">
         <v>141</v>
       </c>
-      <c r="D413" s="29"/>
-    </row>
-    <row r="414" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A414" s="31" t="s">
+      <c r="D425" s="29"/>
+    </row>
+    <row r="426" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A426" s="31" t="s">
         <v>533</v>
       </c>
-      <c r="B414" s="28" t="s">
+      <c r="B426" s="28" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="415" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A415" s="28" t="s">
+    <row r="427" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A427" s="28" t="s">
         <v>534</v>
       </c>
-      <c r="B415" s="28" t="s">
+      <c r="B427" s="28" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="416" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A416" s="32" t="s">
+    <row r="428" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A428" s="32" t="s">
         <v>535</v>
       </c>
-      <c r="B416" s="28" t="s">
+      <c r="B428" s="28" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="417" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A417" s="31" t="s">
+    <row r="429" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A429" s="31" t="s">
         <v>527</v>
       </c>
-      <c r="B417" s="28" t="s">
+      <c r="B429" s="28" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="418" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A418" s="31" t="s">
+    <row r="430" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A430" s="31" t="s">
         <v>529</v>
       </c>
-      <c r="B418" s="28" t="s">
+      <c r="B430" s="28" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="419" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A419" s="10" t="s">
+    <row r="431" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A431" s="10" t="s">
         <v>540</v>
       </c>
-      <c r="B419" s="28" t="s">
+      <c r="B431" s="28" t="s">
         <v>141</v>
       </c>
-      <c r="C419" s="2"/>
-    </row>
-    <row r="420" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A420" s="31" t="s">
+      <c r="C431" s="2"/>
+    </row>
+    <row r="432" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A432" s="31" t="s">
         <v>528</v>
       </c>
-      <c r="B420" s="28" t="s">
+      <c r="B432" s="28" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="421" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A421" s="32" t="s">
+    <row r="433" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A433" s="32" t="s">
         <v>536</v>
       </c>
-      <c r="B421" s="28" t="s">
+      <c r="B433" s="28" t="s">
         <v>141</v>
       </c>
-      <c r="C421" s="10"/>
-    </row>
-    <row r="422" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A422" s="28" t="s">
+      <c r="C433" s="10"/>
+    </row>
+    <row r="434" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A434" s="28" t="s">
         <v>521</v>
       </c>
-      <c r="B422" s="28" t="s">
+      <c r="B434" s="28" t="s">
         <v>141</v>
       </c>
-      <c r="C422" s="28"/>
-      <c r="D422" s="29"/>
-    </row>
-    <row r="423" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A423" s="2" t="s">
+      <c r="C434" s="28"/>
+      <c r="D434" s="29"/>
+    </row>
+    <row r="435" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A435" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="B423" s="2" t="s">
+      <c r="B435" s="2" t="s">
         <v>542</v>
       </c>
-      <c r="C423" s="2" t="s">
+      <c r="C435" s="2" t="s">
         <v>523</v>
       </c>
     </row>
-    <row r="424" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A424" s="2" t="s">
+    <row r="436" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A436" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B424" s="2" t="s">
+      <c r="B436" s="2" t="s">
         <v>542</v>
       </c>
-      <c r="C424" s="2" t="s">
+      <c r="C436" s="2" t="s">
         <v>524</v>
       </c>
     </row>
-    <row r="425" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A425" s="2" t="s">
+    <row r="437" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A437" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B425" s="2" t="s">
+      <c r="B437" s="2" t="s">
         <v>542</v>
       </c>
-      <c r="C425" s="2" t="s">
+      <c r="C437" s="2" t="s">
         <v>525</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update protocol schema and TOR template
Replace inst/resources/protocol_schema_iphra.xlsx and inst/resources/reach_tor_iphra_template.docx with updated binary versions. These updates refresh the protocol schema spreadsheet and the TOR/template document used in IPHRA workflows; no source code changes.
</commit_message>
<xml_diff>
--- a/inst/resources/protocol_schema_iphra.xlsx
+++ b/inst/resources/protocol_schema_iphra.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R Projects\SaeedR1987\public_health_resources\inst\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7977D509-C76A-44CF-A89E-AFB9B54262F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5B5D175-2FF5-41FB-B51E-8968E44ABDEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1147" uniqueCount="693">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1273" uniqueCount="765">
   <si>
     <t>tag_name</t>
   </si>
@@ -2238,12 +2238,229 @@
   <si>
     <t>@total_population_size</t>
   </si>
+  <si>
+    <t>@total_population_size_strata</t>
+  </si>
+  <si>
+    <t>@inc_muac_children</t>
+  </si>
+  <si>
+    <t>@inc_iycfe</t>
+  </si>
+  <si>
+    <t>@inc_muac_plw</t>
+  </si>
+  <si>
+    <t>@inc_cdr</t>
+  </si>
+  <si>
+    <t>@inc_u5dr</t>
+  </si>
+  <si>
+    <t>ind_muac_children</t>
+  </si>
+  <si>
+    <t>ind_iycfe</t>
+  </si>
+  <si>
+    <t>ind_cdr</t>
+  </si>
+  <si>
+    <t>ind_u5dr</t>
+  </si>
+  <si>
+    <t>ind_muac_plw</t>
+  </si>
+  <si>
+    <t>@inc_ecfies</t>
+  </si>
+  <si>
+    <t>ind_ecfies</t>
+  </si>
+  <si>
+    <t>@inc_measles_vaccination</t>
+  </si>
+  <si>
+    <t>@inc_vitamin_a_coverage</t>
+  </si>
+  <si>
+    <t>ind_measles_vaccination</t>
+  </si>
+  <si>
+    <t>ind_vitamin_a_coverage</t>
+  </si>
+  <si>
+    <t>@text_ind_muac_children</t>
+  </si>
+  <si>
+    <t>@text_ind_muac_plw</t>
+  </si>
+  <si>
+    <t>@text_ind_measles_vaccination</t>
+  </si>
+  <si>
+    <t>@text_ind_vitamin_a_coverage</t>
+  </si>
+  <si>
+    <t>@text_ind_ecfies</t>
+  </si>
+  <si>
+    <t>@text_ind_iycfe</t>
+  </si>
+  <si>
+    <t>@text_ind_cdr</t>
+  </si>
+  <si>
+    <t>@text_ind_u5dr</t>
+  </si>
+  <si>
+    <t>All sampled households within the target population</t>
+  </si>
+  <si>
+    <t>All children 6-59 months of age within sampled households</t>
+  </si>
+  <si>
+    <t>All children 9-59 months of age within sampled households</t>
+  </si>
+  <si>
+    <t>All children 0-23 months of age within sampled households</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All women 15-49 years of age that are pregnant or breastfeeding a child 0-5 months of age within sampled households </t>
+  </si>
+  <si>
+    <t>All individuals within sampled households</t>
+  </si>
+  <si>
+    <t>@header_poptable_population</t>
+  </si>
+  <si>
+    <t>@header_poptable_indicator</t>
+  </si>
+  <si>
+    <t>Indicator(s)</t>
+  </si>
+  <si>
+    <t>Population</t>
+  </si>
+  <si>
+    <t>@text_ind_general_population</t>
+  </si>
+  <si>
+    <t>General Household Indicators</t>
+  </si>
+  <si>
+    <t>@text_indname_general</t>
+  </si>
+  <si>
+    <t>@text_indname_muac_children</t>
+  </si>
+  <si>
+    <t>@text_indname_vitamin_a_coverage</t>
+  </si>
+  <si>
+    <t>@text_indname_ecfies</t>
+  </si>
+  <si>
+    <t>@text_indname_iycfe</t>
+  </si>
+  <si>
+    <t>@text_indname_muac_plw</t>
+  </si>
+  <si>
+    <t>@text_indname_cdr</t>
+  </si>
+  <si>
+    <t>@text_indname_u5dr</t>
+  </si>
+  <si>
+    <t>Global Acute Malnutrition by MUAC</t>
+  </si>
+  <si>
+    <t>Measles Vaccination Coverage</t>
+  </si>
+  <si>
+    <t>Vitamin A Supplementation Coverage</t>
+  </si>
+  <si>
+    <t>Early Childhood Food Insecurity Scale (ECFIES)</t>
+  </si>
+  <si>
+    <t>Infant and Young Child Feeding in Emergencies (IYCF-E) Questions</t>
+  </si>
+  <si>
+    <t>Global Acute Malnutrition by MUAC for Pregnant and Lactating Women</t>
+  </si>
+  <si>
+    <t>Crude Death Rate</t>
+  </si>
+  <si>
+    <t>Under-5 Death Rate</t>
+  </si>
+  <si>
+    <t>@text_population_of_interest</t>
+  </si>
+  <si>
+    <t>@text_population_strata</t>
+  </si>
+  <si>
+    <t>multiple_strata</t>
+  </si>
+  <si>
+    <t>This assessment will assess @total_population_size_strata .</t>
+  </si>
+  <si>
+    <t>@text_indname_measles_vaccination</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The population of interest is @total_population_size people. @text_population_strata . @geographic_coverage .
+Within this population, specific indicators will target sub-populations, including: </t>
+  </si>
+  <si>
+    <t>@header_household_surveys</t>
+  </si>
+  <si>
+    <t>@header_sample_size</t>
+  </si>
+  <si>
+    <t>Household surveys</t>
+  </si>
+  <si>
+    <t>Sample Size</t>
+  </si>
+  <si>
+    <t>@header_site_selection_methods</t>
+  </si>
+  <si>
+    <t>Site Selection Methods</t>
+  </si>
+  <si>
+    <t>@text_site_selection_srs</t>
+  </si>
+  <si>
+    <t>@text_site_selection_systematic</t>
+  </si>
+  <si>
+    <t>@site_selection_exhaustive</t>
+  </si>
+  <si>
+    <t>@site_selection_purposive</t>
+  </si>
+  <si>
+    <t>@text_site_selection_cluster</t>
+  </si>
+  <si>
+    <t>@text_site_selection_noncluster</t>
+  </si>
+  <si>
+    <t>Due to a lack of reliable population data, sites will be selected with simple random sampling with each site having an equal change of selection.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2401,6 +2618,12 @@
       <name val="Arial Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -2428,7 +2651,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -2490,6 +2713,13 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2793,7 +3023,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D437"/>
+  <dimension ref="A1:D467"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="53.140625" customWidth="1"/>
@@ -6771,430 +7001,858 @@
         <v>691</v>
       </c>
     </row>
-    <row r="392" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:4" ht="66" x14ac:dyDescent="0.25">
       <c r="A392" s="2" t="s">
+        <v>746</v>
+      </c>
+      <c r="B392" t="s">
+        <v>140</v>
+      </c>
+      <c r="C392" s="2"/>
+      <c r="D392" s="40" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="393" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A393" s="2" t="s">
         <v>692</v>
       </c>
-      <c r="B392" t="s">
+      <c r="B393" t="s">
         <v>141</v>
       </c>
-      <c r="C392" s="2"/>
-      <c r="D392" s="27"/>
-    </row>
-    <row r="393" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A393" s="2"/>
       <c r="C393" s="2"/>
       <c r="D393" s="27"/>
     </row>
     <row r="394" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A394" s="2"/>
-      <c r="C394" s="2"/>
-      <c r="D394" s="27"/>
+      <c r="A394" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="B394" t="s">
+        <v>140</v>
+      </c>
+      <c r="C394" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="D394" s="27" t="s">
+        <v>749</v>
+      </c>
     </row>
     <row r="395" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A395" s="2"/>
+      <c r="A395" s="2" t="s">
+        <v>693</v>
+      </c>
+      <c r="B395" t="s">
+        <v>141</v>
+      </c>
       <c r="C395" s="2"/>
       <c r="D395" s="27"/>
     </row>
     <row r="396" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A396" s="2"/>
-      <c r="C396" s="2"/>
+      <c r="A396" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="B396" t="s">
+        <v>302</v>
+      </c>
+      <c r="C396" s="2" t="s">
+        <v>699</v>
+      </c>
       <c r="D396" s="27"/>
     </row>
     <row r="397" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A397" s="2"/>
-      <c r="C397" s="2"/>
+      <c r="A397" s="2" t="s">
+        <v>706</v>
+      </c>
+      <c r="B397" t="s">
+        <v>302</v>
+      </c>
+      <c r="C397" s="2" t="s">
+        <v>708</v>
+      </c>
       <c r="D397" s="27"/>
     </row>
     <row r="398" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A398" s="2"/>
-      <c r="C398" s="2"/>
+      <c r="A398" s="2" t="s">
+        <v>707</v>
+      </c>
+      <c r="B398" t="s">
+        <v>302</v>
+      </c>
+      <c r="C398" s="2" t="s">
+        <v>709</v>
+      </c>
       <c r="D398" s="27"/>
     </row>
     <row r="399" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A399" s="2"/>
-      <c r="C399" s="2"/>
+      <c r="A399" s="2" t="s">
+        <v>704</v>
+      </c>
+      <c r="B399" t="s">
+        <v>302</v>
+      </c>
+      <c r="C399" s="2" t="s">
+        <v>705</v>
+      </c>
       <c r="D399" s="27"/>
     </row>
     <row r="400" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A400" s="2"/>
-      <c r="C400" s="2"/>
+      <c r="A400" s="2" t="s">
+        <v>695</v>
+      </c>
+      <c r="B400" t="s">
+        <v>302</v>
+      </c>
+      <c r="C400" s="2" t="s">
+        <v>700</v>
+      </c>
       <c r="D400" s="27"/>
     </row>
     <row r="401" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A401" s="2"/>
-      <c r="C401" s="2"/>
+      <c r="A401" s="2" t="s">
+        <v>696</v>
+      </c>
+      <c r="B401" t="s">
+        <v>302</v>
+      </c>
+      <c r="C401" s="2" t="s">
+        <v>703</v>
+      </c>
       <c r="D401" s="27"/>
     </row>
     <row r="402" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A402" s="2"/>
-      <c r="C402" s="2"/>
+      <c r="A402" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="B402" t="s">
+        <v>302</v>
+      </c>
+      <c r="C402" s="2" t="s">
+        <v>701</v>
+      </c>
       <c r="D402" s="27"/>
     </row>
     <row r="403" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A403" s="2"/>
-      <c r="C403" s="2"/>
+      <c r="A403" s="2" t="s">
+        <v>698</v>
+      </c>
+      <c r="B403" t="s">
+        <v>302</v>
+      </c>
+      <c r="C403" s="2" t="s">
+        <v>702</v>
+      </c>
       <c r="D403" s="27"/>
     </row>
-    <row r="404" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A404" s="2"/>
+    <row r="404" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A404" s="2" t="s">
+        <v>725</v>
+      </c>
+      <c r="B404" t="s">
+        <v>140</v>
+      </c>
       <c r="C404" s="2"/>
-      <c r="D404" s="27"/>
-    </row>
-    <row r="406" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D404" s="26" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="405" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A405" s="2" t="s">
+        <v>724</v>
+      </c>
+      <c r="B405" t="s">
+        <v>140</v>
+      </c>
+      <c r="C405" s="2"/>
+      <c r="D405" s="26" t="s">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="406" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A406" s="2" t="s">
-        <v>549</v>
+        <v>730</v>
       </c>
       <c r="B406" t="s">
         <v>140</v>
       </c>
-      <c r="D406" s="26" t="s">
-        <v>551</v>
-      </c>
-    </row>
-    <row r="407" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="C406" s="2"/>
+      <c r="D406" s="38" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="407" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A407" s="2" t="s">
-        <v>550</v>
+        <v>731</v>
       </c>
       <c r="B407" t="s">
         <v>140</v>
       </c>
-      <c r="D407" s="27" t="s">
-        <v>552</v>
+      <c r="C407" s="2" t="s">
+        <v>699</v>
+      </c>
+      <c r="D407" s="39" t="s">
+        <v>738</v>
       </c>
     </row>
     <row r="408" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A408" t="s">
-        <v>114</v>
+      <c r="A408" s="2" t="s">
+        <v>750</v>
       </c>
       <c r="B408" t="s">
-        <v>511</v>
+        <v>140</v>
+      </c>
+      <c r="C408" s="2" t="s">
+        <v>708</v>
+      </c>
+      <c r="D408" s="39" t="s">
+        <v>739</v>
       </c>
     </row>
     <row r="409" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A409" s="2" t="s">
-        <v>553</v>
+        <v>732</v>
       </c>
       <c r="B409" t="s">
         <v>140</v>
       </c>
-      <c r="D409" t="s">
-        <v>554</v>
+      <c r="C409" s="2" t="s">
+        <v>709</v>
+      </c>
+      <c r="D409" s="39" t="s">
+        <v>740</v>
       </c>
     </row>
     <row r="410" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A410" t="s">
-        <v>115</v>
+      <c r="A410" s="2" t="s">
+        <v>733</v>
       </c>
       <c r="B410" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="411" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+      <c r="C410" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="D410" s="39" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="411" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A411" s="2" t="s">
-        <v>547</v>
+        <v>734</v>
       </c>
       <c r="B411" t="s">
         <v>140</v>
       </c>
-      <c r="D411" s="33" t="s">
-        <v>548</v>
+      <c r="C411" s="2" t="s">
+        <v>700</v>
+      </c>
+      <c r="D411" s="39" t="s">
+        <v>742</v>
       </c>
     </row>
     <row r="412" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A412" s="2" t="s">
-        <v>128</v>
+        <v>735</v>
       </c>
       <c r="B412" t="s">
-        <v>499</v>
+        <v>140</v>
       </c>
       <c r="C412" s="2" t="s">
-        <v>513</v>
-      </c>
-      <c r="D412" t="s">
-        <v>129</v>
+        <v>703</v>
+      </c>
+      <c r="D412" s="39" t="s">
+        <v>743</v>
       </c>
     </row>
     <row r="413" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A413" s="2" t="s">
-        <v>116</v>
+        <v>736</v>
       </c>
       <c r="B413" t="s">
-        <v>499</v>
+        <v>140</v>
       </c>
       <c r="C413" s="2" t="s">
-        <v>519</v>
-      </c>
-      <c r="D413" t="s">
-        <v>122</v>
+        <v>701</v>
+      </c>
+      <c r="D413" s="39" t="s">
+        <v>744</v>
       </c>
     </row>
     <row r="414" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A414" s="2" t="s">
-        <v>126</v>
+        <v>737</v>
       </c>
       <c r="B414" t="s">
-        <v>499</v>
+        <v>140</v>
       </c>
       <c r="C414" s="2" t="s">
-        <v>514</v>
-      </c>
-      <c r="D414" t="s">
-        <v>127</v>
+        <v>702</v>
+      </c>
+      <c r="D414" s="39" t="s">
+        <v>745</v>
       </c>
     </row>
     <row r="415" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A415" s="2" t="s">
-        <v>117</v>
+        <v>728</v>
       </c>
       <c r="B415" t="s">
-        <v>499</v>
-      </c>
-      <c r="C415" s="2" t="s">
-        <v>515</v>
-      </c>
-      <c r="D415" t="s">
-        <v>121</v>
+        <v>140</v>
+      </c>
+      <c r="C415" s="2"/>
+      <c r="D415" s="38" t="s">
+        <v>718</v>
       </c>
     </row>
     <row r="416" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A416" s="2" t="s">
-        <v>118</v>
+        <v>710</v>
       </c>
       <c r="B416" t="s">
-        <v>499</v>
+        <v>140</v>
       </c>
       <c r="C416" s="2" t="s">
-        <v>516</v>
-      </c>
-      <c r="D416" t="s">
-        <v>123</v>
+        <v>699</v>
+      </c>
+      <c r="D416" s="2" t="s">
+        <v>718</v>
       </c>
     </row>
     <row r="417" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A417" s="2" t="s">
-        <v>119</v>
+        <v>712</v>
       </c>
       <c r="B417" t="s">
-        <v>499</v>
+        <v>140</v>
       </c>
       <c r="C417" s="2" t="s">
-        <v>517</v>
-      </c>
-      <c r="D417" t="s">
-        <v>125</v>
+        <v>708</v>
+      </c>
+      <c r="D417" s="2" t="s">
+        <v>719</v>
       </c>
     </row>
     <row r="418" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A418" s="2" t="s">
-        <v>120</v>
+        <v>713</v>
       </c>
       <c r="B418" t="s">
-        <v>499</v>
+        <v>140</v>
       </c>
       <c r="C418" s="2" t="s">
-        <v>518</v>
-      </c>
-      <c r="D418" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="419" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+        <v>709</v>
+      </c>
+      <c r="D418" s="2" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="419" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A419" s="2" t="s">
-        <v>543</v>
+        <v>714</v>
       </c>
       <c r="B419" t="s">
         <v>140</v>
       </c>
-      <c r="C419" s="2"/>
-      <c r="D419" s="26" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="420" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="C419" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="D419" s="2" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="420" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A420" s="2" t="s">
-        <v>545</v>
+        <v>715</v>
       </c>
       <c r="B420" t="s">
         <v>140</v>
       </c>
-      <c r="C420" s="2"/>
-      <c r="D420" s="10" t="s">
-        <v>546</v>
+      <c r="C420" s="2" t="s">
+        <v>700</v>
+      </c>
+      <c r="D420" s="2" t="s">
+        <v>721</v>
       </c>
     </row>
     <row r="421" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A421" s="2" t="s">
-        <v>522</v>
+        <v>711</v>
       </c>
       <c r="B421" t="s">
-        <v>499</v>
+        <v>140</v>
       </c>
       <c r="C421" s="2" t="s">
-        <v>523</v>
-      </c>
-      <c r="D421" t="s">
-        <v>526</v>
+        <v>703</v>
+      </c>
+      <c r="D421" s="2" t="s">
+        <v>721</v>
       </c>
     </row>
     <row r="422" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A422" s="2" t="s">
-        <v>530</v>
+        <v>716</v>
       </c>
       <c r="B422" t="s">
+        <v>140</v>
+      </c>
+      <c r="C422" s="2" t="s">
+        <v>701</v>
+      </c>
+      <c r="D422" s="2" t="s">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="423" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A423" s="2" t="s">
+        <v>717</v>
+      </c>
+      <c r="B423" t="s">
+        <v>140</v>
+      </c>
+      <c r="C423" s="2" t="s">
+        <v>702</v>
+      </c>
+      <c r="D423" s="2" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="424" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A424" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="B424" t="s">
+        <v>140</v>
+      </c>
+      <c r="D424" s="26" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="425" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A425" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="B425" t="s">
+        <v>140</v>
+      </c>
+      <c r="D425" s="27" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="426" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A426" t="s">
+        <v>114</v>
+      </c>
+      <c r="B426" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="427" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A427" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="B427" t="s">
+        <v>140</v>
+      </c>
+      <c r="D427" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="428" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A428" t="s">
+        <v>115</v>
+      </c>
+      <c r="B428" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="429" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A429" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="B429" t="s">
+        <v>140</v>
+      </c>
+      <c r="D429" s="33" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="430" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A430" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B430" t="s">
         <v>499</v>
       </c>
-      <c r="C422" s="2" t="s">
-        <v>524</v>
-      </c>
-      <c r="D422" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="423" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A423" s="30" t="s">
-        <v>537</v>
-      </c>
-      <c r="B423" t="s">
+      <c r="C430" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="D430" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="431" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A431" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B431" t="s">
         <v>499</v>
       </c>
-      <c r="C423" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="D423" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="424" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A424" s="30" t="s">
-        <v>538</v>
-      </c>
-      <c r="B424" t="s">
+      <c r="C431" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="D431" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="432" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A432" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B432" t="s">
         <v>499</v>
       </c>
-      <c r="C424" s="2" t="s">
-        <v>531</v>
-      </c>
-      <c r="D424" t="s">
-        <v>541</v>
-      </c>
-    </row>
-    <row r="425" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A425" s="28" t="s">
-        <v>520</v>
-      </c>
-      <c r="B425" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="D425" s="29"/>
-    </row>
-    <row r="426" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A426" s="31" t="s">
-        <v>533</v>
-      </c>
-      <c r="B426" s="28" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="427" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A427" s="28" t="s">
-        <v>534</v>
-      </c>
-      <c r="B427" s="28" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="428" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A428" s="32" t="s">
-        <v>535</v>
-      </c>
-      <c r="B428" s="28" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="429" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A429" s="31" t="s">
-        <v>527</v>
-      </c>
-      <c r="B429" s="28" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="430" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A430" s="31" t="s">
-        <v>529</v>
-      </c>
-      <c r="B430" s="28" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="431" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A431" s="10" t="s">
-        <v>540</v>
-      </c>
-      <c r="B431" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="C431" s="2"/>
-    </row>
-    <row r="432" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A432" s="31" t="s">
-        <v>528</v>
-      </c>
-      <c r="B432" s="28" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="433" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A433" s="32" t="s">
-        <v>536</v>
-      </c>
-      <c r="B433" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="C433" s="10"/>
+      <c r="C432" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="D432" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="433" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A433" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B433" t="s">
+        <v>499</v>
+      </c>
+      <c r="C433" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="D433" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="434" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A434" s="28" t="s">
-        <v>521</v>
-      </c>
-      <c r="B434" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="C434" s="28"/>
-      <c r="D434" s="29"/>
+      <c r="A434" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B434" t="s">
+        <v>499</v>
+      </c>
+      <c r="C434" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="D434" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="435" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A435" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="B435" s="2" t="s">
-        <v>542</v>
+        <v>119</v>
+      </c>
+      <c r="B435" t="s">
+        <v>499</v>
       </c>
       <c r="C435" s="2" t="s">
-        <v>523</v>
+        <v>517</v>
+      </c>
+      <c r="D435" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="436" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A436" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B436" t="s">
+        <v>499</v>
+      </c>
+      <c r="C436" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="D436" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="437" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A437" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="B437" t="s">
+        <v>140</v>
+      </c>
+      <c r="C437" s="2"/>
+      <c r="D437" s="26" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="438" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A438" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="B438" t="s">
+        <v>140</v>
+      </c>
+      <c r="C438" s="2"/>
+      <c r="D438" s="10" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="439" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A439" s="2" t="s">
+        <v>752</v>
+      </c>
+      <c r="B439" t="s">
+        <v>140</v>
+      </c>
+      <c r="C439" s="2"/>
+      <c r="D439" s="10" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="440" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A440" s="2" t="s">
+        <v>753</v>
+      </c>
+      <c r="B440" t="s">
+        <v>140</v>
+      </c>
+      <c r="C440" s="2"/>
+      <c r="D440" s="10" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="441" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A441" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="B441" t="s">
+        <v>499</v>
+      </c>
+      <c r="C441" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="D441" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="442" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A442" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="B442" t="s">
+        <v>499</v>
+      </c>
+      <c r="C442" s="2" t="s">
+        <v>524</v>
+      </c>
+      <c r="D442" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="443" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A443" s="30" t="s">
+        <v>537</v>
+      </c>
+      <c r="B443" t="s">
+        <v>499</v>
+      </c>
+      <c r="C443" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="D443" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="444" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A444" s="30" t="s">
+        <v>538</v>
+      </c>
+      <c r="B444" t="s">
+        <v>499</v>
+      </c>
+      <c r="C444" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="D444" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="445" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A445" s="28" t="s">
+        <v>520</v>
+      </c>
+      <c r="B445" s="28" t="s">
+        <v>141</v>
+      </c>
+      <c r="D445" s="29"/>
+    </row>
+    <row r="446" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A446" s="31" t="s">
+        <v>533</v>
+      </c>
+      <c r="B446" s="28" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="447" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A447" s="28" t="s">
+        <v>534</v>
+      </c>
+      <c r="B447" s="28" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="448" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A448" s="32" t="s">
+        <v>535</v>
+      </c>
+      <c r="B448" s="28" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="449" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A449" s="31" t="s">
+        <v>527</v>
+      </c>
+      <c r="B449" s="28" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="450" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A450" s="31" t="s">
+        <v>529</v>
+      </c>
+      <c r="B450" s="28" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="451" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A451" s="10" t="s">
+        <v>540</v>
+      </c>
+      <c r="B451" s="28" t="s">
+        <v>141</v>
+      </c>
+      <c r="C451" s="2"/>
+    </row>
+    <row r="452" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A452" s="31" t="s">
+        <v>528</v>
+      </c>
+      <c r="B452" s="28" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="453" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A453" s="32" t="s">
+        <v>536</v>
+      </c>
+      <c r="B453" s="28" t="s">
+        <v>141</v>
+      </c>
+      <c r="C453" s="10"/>
+    </row>
+    <row r="454" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A454" s="28" t="s">
+        <v>521</v>
+      </c>
+      <c r="B454" s="28" t="s">
+        <v>141</v>
+      </c>
+      <c r="C454" s="28"/>
+      <c r="D454" s="29"/>
+    </row>
+    <row r="455" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A455" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B455" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="C455" s="2" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="456" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A456" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B436" s="2" t="s">
+      <c r="B456" s="2" t="s">
         <v>542</v>
       </c>
-      <c r="C436" s="2" t="s">
+      <c r="C456" s="2" t="s">
         <v>524</v>
       </c>
     </row>
-    <row r="437" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A437" s="2" t="s">
+    <row r="457" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A457" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B437" s="2" t="s">
+      <c r="B457" s="2" t="s">
         <v>542</v>
       </c>
-      <c r="C437" s="2" t="s">
+      <c r="C457" s="2" t="s">
         <v>525</v>
+      </c>
+    </row>
+    <row r="458" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A458" s="2"/>
+      <c r="C458" s="2"/>
+      <c r="D458" s="10"/>
+    </row>
+    <row r="459" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A459" s="2" t="s">
+        <v>756</v>
+      </c>
+      <c r="B459" t="s">
+        <v>140</v>
+      </c>
+      <c r="C459" s="2"/>
+      <c r="D459" s="10" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="460" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A460" s="2"/>
+      <c r="C460" s="2"/>
+      <c r="D460" s="10"/>
+    </row>
+    <row r="461" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A461" s="2" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="462" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A462" s="2" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="463" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A463" s="2" t="s">
+        <v>758</v>
+      </c>
+      <c r="D463" s="10" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="464" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A464" s="2" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="465" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A465" s="2" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="466" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A466" s="2" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="467" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A467" s="2" t="s">
+        <v>761</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update iPHRA protocol schema and TOR template
Refresh binary resource files used by iPHRA: update inst/resources/protocol_schema_iphra.xlsx and inst/resources/reach_tor_iphra_template.docx with content/formatting changes. These are asset updates only and do not modify source code.
</commit_message>
<xml_diff>
--- a/inst/resources/protocol_schema_iphra.xlsx
+++ b/inst/resources/protocol_schema_iphra.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saeed.rahman\Desktop\public_health_resources\inst\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R Projects\SaeedR1987\public_health_resources\inst\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DA6647F-01F9-4D99-9E7E-337BD841E90F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{835BF67D-99B0-49B8-99A6-0DE7E5559656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="schema" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1555" uniqueCount="936">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1618" uniqueCount="986">
   <si>
     <t>tag_name</t>
   </si>
@@ -1708,12 +1708,6 @@
     <t>definition_muac</t>
   </si>
   <si>
-    <t>definition_cdr</t>
-  </si>
-  <si>
-    <t>definition_u5dr</t>
-  </si>
-  <si>
     <t>definition_complementary_feeding</t>
   </si>
   <si>
@@ -2240,12 +2234,6 @@
   </si>
   <si>
     <t>ind_iycfe</t>
-  </si>
-  <si>
-    <t>ind_cdr</t>
-  </si>
-  <si>
-    <t>ind_u5dr</t>
   </si>
   <si>
     <t>ind_muac_plw</t>
@@ -3048,6 +3036,175 @@
   </si>
   <si>
     <t>Crop/Livestock observations (Target #):</t>
+  </si>
+  <si>
+    <t>@num_enumerators_per_team</t>
+  </si>
+  <si>
+    <t>@num_days_data_collection</t>
+  </si>
+  <si>
+    <t>@text_training_mortality</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A dedicated session on collecting mortality data will be included. </t>
+  </si>
+  <si>
+    <t>@text_training_muac</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An additional session will be included for training on MUAC measurements as well as a half day of training for a MUAC standardization test. </t>
+  </si>
+  <si>
+    <t>Team Composition, Training, and Quality Assurance</t>
+  </si>
+  <si>
+    <t>The exact composition of teams will depend on the number of tools being implemented. For household surveys, teams will consist of one field supervisor and @num_enumerators_per_team enumerators (@num_enumerators_per_team enumerators : 1 ratio). Where possible, teams should incorporate a mix of male and female enumerators. For key informant and observational tools, dedicated enumerators separate from the household survey enumerators will be selected and trained to implement them. One enumerator should not implement more than one or two specific tools to ensure adequate time for use in the field and data quality. 
+Teams will receive a base three-day training prior to data collection covering purpose of the survey, good interview practices and ethical conduct during public health assessment, field sampling procedures, and review of the survey, key informant and observational tools, and a one-day for pilot and planning activities. @text_training_mortality It is recommended to divide the team for separate tool review sessions to efficiently make use of training time. @text_training_muac 
+Field supervisors will have a key role in ensuring research quality during data collection. Key responsibilities will include:
+-	Providing daily feedback sessions to the data collection team
+-	Monitoring completion of assessment against planned targets
+-	Completing cluster control forms
+-	Ensuring proper household sampling techniques are applied
+-	Providing supportive supervision to enumerators</t>
+  </si>
+  <si>
+    <t>@header_team_comp_quality</t>
+  </si>
+  <si>
+    <t>@text_team_comp_quality</t>
+  </si>
+  <si>
+    <t>@header_data_collection_plan</t>
+  </si>
+  <si>
+    <t>Data Collection Plan</t>
+  </si>
+  <si>
+    <t>@text_intro_data_collection_plan</t>
+  </si>
+  <si>
+    <t>@data_collection_plan_table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The below table summarizes the planning assumptions for the household survey component of the IPHRA and the estimate for days needed to complete the assessment. Key informant and observation tools will be conducted simultaneously to the household survey. Overall, data collection will be conducted for @num_days_data_collection.   </t>
+  </si>
+  <si>
+    <t>mortality_survey</t>
+  </si>
+  <si>
+    <t>Household Survey</t>
+  </si>
+  <si>
+    <t>Data Processing &amp; Analysis</t>
+  </si>
+  <si>
+    <t>@header_data_processing_analysis</t>
+  </si>
+  <si>
+    <t>@header_kii_obs_analysis</t>
+  </si>
+  <si>
+    <t>@header_household_survey_analysis</t>
+  </si>
+  <si>
+    <t>@header_integrated_analysis</t>
+  </si>
+  <si>
+    <t>@text_analysis_exhaustive_srs_systematic_unstratified</t>
+  </si>
+  <si>
+    <t>The finite population correction factor will be applied since the target population is less than 10,000 individuals.</t>
+  </si>
+  <si>
+    <t>@text_analysis_fpc_unstratified</t>
+  </si>
+  <si>
+    <t>For specific stratum where the population is less than 10,000 individuals, the finite population correction factor will be applied.</t>
+  </si>
+  <si>
+    <t>@text_analysis_fpc_stratified</t>
+  </si>
+  <si>
+    <t>Data will be collected using a contextualized IPHRA ODK tool. Cleaning and analysis will be done using a pre-prepared IPHRA application built in @r_version.</t>
+  </si>
+  <si>
+    <t>@text_intro_data_processing_analysis</t>
+  </si>
+  <si>
+    <t>The household analysis will be treated as a simple random sampling design across sites without applying survey weights. @text_analysis_fpc_unstratified.</t>
+  </si>
+  <si>
+    <t>@text_analysis_exhaustive_srs_systematic_stratified</t>
+  </si>
+  <si>
+    <t>The household analysis will be treated as a simple random sampling design across sites. Survey weights will be generated for aggregation of results between strata. @text_analysis_fpc_stratified</t>
+  </si>
+  <si>
+    <t>@text_analysis_srs_systematic_srs_systematic_stratified</t>
+  </si>
+  <si>
+    <t>@text_analysis_srs_systematic_srs_systematic_unstratified</t>
+  </si>
+  <si>
+    <t>The household analysis will be treated as a weighted analysis and survey weights will be generated between sites to correct for under- or over-sampling between sites based on the best available population estimated the field teams were able to recover. If no adequate population data was available during the assessment, the final analysis will be unweighted. @text_analysis_fpc_unstratified</t>
+  </si>
+  <si>
+    <t>The household analysis will be treated as a weighted analysis and survey weights will be generated between sites to correct for under- or over-sampling between sites based on the best available population estimated the field teams were able to recover. If no adequate population data was available during the assessment, the final analysis will be unweighted. An additional set of weights will be generated between strata to account for under- or over-sampling of population groups. Each set of weights will be multiplied together at the household level to generate a single set of composite weights for aggregated analysis. @text_analysis_fpc_stratified</t>
+  </si>
+  <si>
+    <t>@text_analysis_cluster_srs_systematic_unstratified</t>
+  </si>
+  <si>
+    <t>The household analysis will be treated as a cluster design without applying survey weights. Sites/PSUs will be treated as clusters in the analysis. @text_analysis_fpc_unstratified</t>
+  </si>
+  <si>
+    <t>@text_analysis_cluster_srs_systematic_stratified</t>
+  </si>
+  <si>
+    <t>The household analysis will be treated as a cluster design and sites/PSUs will be treated as clusters in the analysis. Survey weights will be generated for aggregation of results between strata. @text_analysis_fpc_stratified</t>
+  </si>
+  <si>
+    <t>@text_analysis_exhaustive_rlc_unstratified</t>
+  </si>
+  <si>
+    <t>The household analysis will be treated as a cluster design across sites with groupings of households at each GPS point treated as the clusters in the analysis. If population density is assessed to be very different within or across assessment sites, survey weights will be used for each random location cluster equivalent to the inverse of the population density of each cluster. This is intended to correct for any bias due to an uneven population density across the assessment area to make sure households have a more equal representation in the dataset. Population density is estimated based on the number of people in households within a random location cluster divided by the area of the circle formed by the locations of the three households and the GPS point of that random location cluster. @text_analysis_fpc_unstratified</t>
+  </si>
+  <si>
+    <t>@text_analysis_exhaustive_rlc_stratified</t>
+  </si>
+  <si>
+    <t>The household analysis will be treated as a cluster design across sites with groupings of households at each GPS point treated as the clusters in the analysis. If population density is assessed to be very different within or across assessment sites, survey weights will be used for each random location cluster equivalent to the inverse of the population density of each cluster. This is intended to correct for any bias due to an uneven population density across the assessment area to make sure households have a more equal representation in the dataset. Population density is estimated based on the number of people in households within a random location cluster divided by the area of the circle formed by the locations of the three households and the GPS point of that random location cluster. An additional set of weights will be generated between strata to account for under- or over-sampling of population groups. Each set of weights will be multiplied together at the household level to generate a single set of composite weights for aggregated analysis. @text_analysis_fpc_stratified</t>
+  </si>
+  <si>
+    <t>@text_analysis_srs_systematic_rlc_unstratified</t>
+  </si>
+  <si>
+    <t>The household analysis will be treated as a weighted cluster design across sites with groupings of households at each GPS point treated as the clusters in the analysis. Survey weights will be generated between sites to correct for under- or over-sampling between sites based on the best available population estimated the field teams were able to recover. If no adequate population data was available during the assessment, the final analysis will be unweighted. If population density is assessed to be very different within or across assessment sites, survey weights will be used for each random location cluster equivalent to the inverse of the population density of each cluster. This is intended to correct for any bias due to an uneven population density across the assessment area to make sure households have a more equal representation in the dataset. Population density is estimated based on the number of people in households within a random location cluster divided by the area of the circle formed by the locations of the three households and the GPS point of that random location cluster. An additional set of weights will be generated between strata to account for under- or over-sampling of population groups. Each set of weights will be multiplied together at the household level to generate a single set of composite weights for aggregated analysis. @text_analysis_fpc_unstratified</t>
+  </si>
+  <si>
+    <t>@text_analysis_srs_systematic_rlc_stratified</t>
+  </si>
+  <si>
+    <t>The household analysis will be treated as a weighted cluster design across sites with groupings of households at each GPS point treated as the clusters in the analysis. Survey weights will be generated between sites to correct for under- or over-sampling between sites based on the best available population estimated the field teams were able to recover. If no adequate population data was available during the assessment, the final analysis will be unweighted. If population density is assessed to be very different within or across assessment sites, survey weights will be used for each random location cluster equivalent to the inverse of the population density of each cluster. This is intended to correct for any bias due to an uneven population density across the assessment area to make sure households have a more equal representation in the dataset. Population density is estimated based on the number of people in households within a random location cluster divided by the area of the circle formed by the locations of the three households and the GPS point of that random location cluster. An additional set of weights will be generated between strata to account for under- or over-sampling of population groups. Each set of weights will be multiplied together at the household level to generate a single set of composite weights for aggregated analysis. @text_analysis_fpc_stratified</t>
+  </si>
+  <si>
+    <t>@text_analysis_cluster_rlc_unstratified</t>
+  </si>
+  <si>
+    <t>The household analysis will be treated as a cluster design with sites/PSU being the primary clusters assigned in the analysis. Within these PSUs, additional clustering effects may be taking place as three households are sampled per random location cluster (GPS point) however this clustering effect will not be explicitly accounted for in the analysis. If population density is assessed to be very different within assessment sites/PSUs, survey weights will be used for each random location cluster equivalent to the inverse of the population density of each random location cluster. This is intended to correct for any bias due to an uneven population density across the assessment area to make sure households have a more equal representation in the dataset. Population density is estimated based on the number of people in households within a random location cluster divided by the area of the circle formed by the locations of the three households and the GPS point of that random location cluster. @text_analysis_fpc_unstratified</t>
+  </si>
+  <si>
+    <t>@text_analysis_cluster_rlc_stratified</t>
+  </si>
+  <si>
+    <t>The household analysis will be treated as a cluster design with sites/PSU being the primary clusters assigned in the analysis. Within these PSUs, additional clustering effects may be taking place as three households are sampled per random location cluster (GPS point) however this clustering effect will not be explicitly accounted for in the analysis. If population density is assessed to be very different within assessment sites/PSUs, survey weights will be used for each random location cluster equivalent to the inverse of the population density of each random location cluster. This is intended to correct for any bias due to an uneven population density across the assessment area to make sure households have a more equal representation in the dataset. Population density is estimated based on the number of people in households within a random location cluster divided by the area of the circle formed by the locations of the three households and the GPS point of that random location cluster. An additional set of weights will be generated between strata to account for under- or over-sampling of population groups. Each set of weights will be multiplied together at the household level to generate a single set of composite weights for aggregated analysis. @text_analysis_fpc_stratified</t>
+  </si>
+  <si>
+    <t>@text_analysis_muac_age_correction</t>
+  </si>
+  <si>
+    <t>The ratio of children 0-23 months of age to children 24-59 months of age in the sample will be evaluated to determine if additional age weighting is needed for analysis of the indicator Global or Severe Acute Malnutrition by MUAC. If strong differences are observed against an expected proportion of two-thirds children 24-59 months out of all under-5 year old children, then a set of weights will be applied if the child is 0-23 months or 24-59 months for this specific indicator. The age weights will be multiplied with any household level weights to generate a single set of composite weight for analysis.</t>
   </si>
 </sst>
 </file>
@@ -3308,7 +3465,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -3378,7 +3535,6 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3398,6 +3554,10 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3701,7 +3861,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D555"/>
+  <dimension ref="A1:D591"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="53.140625" customWidth="1"/>
@@ -6240,18 +6400,18 @@
     </row>
     <row r="266" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A266" s="2" t="s">
-        <v>925</v>
+        <v>921</v>
       </c>
       <c r="B266" t="s">
         <v>140</v>
       </c>
       <c r="D266" s="24" t="s">
-        <v>934</v>
+        <v>930</v>
       </c>
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A267" s="2" t="s">
-        <v>926</v>
+        <v>922</v>
       </c>
       <c r="B267" t="s">
         <v>302</v>
@@ -6259,7 +6419,7 @@
     </row>
     <row r="268" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A268" s="2" t="s">
-        <v>927</v>
+        <v>923</v>
       </c>
       <c r="B268" t="s">
         <v>140</v>
@@ -6270,7 +6430,7 @@
     </row>
     <row r="269" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A269" s="2" t="s">
-        <v>928</v>
+        <v>924</v>
       </c>
       <c r="B269" t="s">
         <v>142</v>
@@ -6278,7 +6438,7 @@
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A270" s="2" t="s">
-        <v>929</v>
+        <v>925</v>
       </c>
       <c r="B270" t="s">
         <v>140</v>
@@ -6289,7 +6449,7 @@
     </row>
     <row r="271" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A271" s="2" t="s">
-        <v>930</v>
+        <v>926</v>
       </c>
       <c r="B271" t="s">
         <v>142</v>
@@ -6297,18 +6457,18 @@
     </row>
     <row r="272" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A272" s="2" t="s">
+        <v>927</v>
+      </c>
+      <c r="B272" t="s">
+        <v>140</v>
+      </c>
+      <c r="D272" s="14" t="s">
         <v>931</v>
-      </c>
-      <c r="B272" t="s">
-        <v>140</v>
-      </c>
-      <c r="D272" s="14" t="s">
-        <v>935</v>
       </c>
     </row>
     <row r="273" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A273" s="2" t="s">
-        <v>932</v>
+        <v>928</v>
       </c>
       <c r="B273" t="s">
         <v>142</v>
@@ -6316,7 +6476,7 @@
     </row>
     <row r="274" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>933</v>
+        <v>929</v>
       </c>
       <c r="B274" t="s">
         <v>171</v>
@@ -6969,7 +7129,7 @@
         <v>499</v>
       </c>
       <c r="C341" s="2" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="D341" s="27" t="s">
         <v>507</v>
@@ -6983,7 +7143,7 @@
         <v>499</v>
       </c>
       <c r="C342" s="2" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="D342" s="27" t="s">
         <v>508</v>
@@ -6997,7 +7157,7 @@
         <v>499</v>
       </c>
       <c r="C343" s="2" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="D343" s="27" t="s">
         <v>509</v>
@@ -7005,30 +7165,30 @@
     </row>
     <row r="344" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A344" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B344" t="s">
         <v>499</v>
       </c>
       <c r="C344" s="2" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="D344" s="27" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="345" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A345" s="2" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="B345" t="s">
         <v>499</v>
       </c>
       <c r="C345" s="2" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="D345" s="27" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="346" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -7039,38 +7199,38 @@
         <v>499</v>
       </c>
       <c r="C346" s="2" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="D346" s="27" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
     </row>
     <row r="347" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A347" s="2" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="B347" t="s">
         <v>499</v>
       </c>
       <c r="C347" s="2" t="s">
-        <v>758</v>
+        <v>754</v>
       </c>
       <c r="D347" s="27" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="348" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A348" s="2" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="B348" t="s">
         <v>499</v>
       </c>
       <c r="C348" s="2" t="s">
-        <v>759</v>
+        <v>755</v>
       </c>
       <c r="D348" s="27" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
     </row>
     <row r="349" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -7081,38 +7241,38 @@
         <v>499</v>
       </c>
       <c r="C349" s="2" t="s">
-        <v>760</v>
+        <v>756</v>
       </c>
       <c r="D349" s="27" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
     </row>
     <row r="350" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A350" s="2" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="B350" t="s">
         <v>499</v>
       </c>
       <c r="C350" s="2" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="D350" s="27" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
     </row>
     <row r="351" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A351" s="2" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="B351" t="s">
         <v>499</v>
       </c>
       <c r="C351" s="2" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="D351" s="27" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="352" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -7123,624 +7283,624 @@
         <v>499</v>
       </c>
       <c r="C352" s="2" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="D352" s="27" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
     </row>
     <row r="353" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A353" s="2" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="B353" t="s">
         <v>499</v>
       </c>
       <c r="C353" s="2" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="D353" s="27" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="354" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A354" s="2" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="B354" t="s">
         <v>499</v>
       </c>
       <c r="C354" s="2" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="D354" s="34" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="355" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A355" s="2" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="B355" t="s">
         <v>499</v>
       </c>
       <c r="C355" s="2" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="D355" s="27" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="356" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A356" s="2" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="B356" t="s">
         <v>499</v>
       </c>
       <c r="C356" s="2" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="D356" s="27" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
     </row>
     <row r="357" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A357" s="35" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="B357" t="s">
         <v>499</v>
       </c>
       <c r="C357" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="D357" s="36" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
     </row>
     <row r="358" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A358" s="35" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="B358" t="s">
         <v>141</v>
       </c>
       <c r="C358" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="D358" s="27"/>
     </row>
     <row r="359" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A359" s="35" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="B359" t="s">
         <v>499</v>
       </c>
       <c r="C359" s="2" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="D359" s="36" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
     </row>
     <row r="360" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A360" s="35" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="B360" t="s">
         <v>141</v>
       </c>
       <c r="C360" s="2" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="D360" s="27"/>
     </row>
     <row r="361" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A361" s="35" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="B361" t="s">
         <v>499</v>
       </c>
       <c r="C361" s="2" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="D361" s="36" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
     </row>
     <row r="362" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A362" s="35" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="B362" t="s">
         <v>141</v>
       </c>
       <c r="C362" s="2" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="D362" s="27"/>
     </row>
     <row r="363" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A363" s="35" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="B363" t="s">
         <v>499</v>
       </c>
       <c r="C363" s="2" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="D363" s="36" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
     </row>
     <row r="364" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A364" s="35" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="B364" t="s">
         <v>141</v>
       </c>
       <c r="C364" s="2" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="D364" s="27"/>
     </row>
     <row r="365" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A365" s="35" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="B365" t="s">
         <v>499</v>
       </c>
       <c r="C365" s="2" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="D365" s="36" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
     </row>
     <row r="366" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A366" s="35" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="B366" t="s">
         <v>141</v>
       </c>
       <c r="C366" s="2" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="D366" s="27"/>
     </row>
     <row r="367" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A367" s="35" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="B367" t="s">
         <v>499</v>
       </c>
       <c r="C367" s="2" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="D367" s="36" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
     </row>
     <row r="368" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A368" s="35" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="B368" t="s">
         <v>141</v>
       </c>
       <c r="C368" s="2" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="D368" s="27"/>
     </row>
     <row r="369" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A369" s="35" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="B369" t="s">
         <v>499</v>
       </c>
       <c r="C369" s="2" t="s">
-        <v>761</v>
+        <v>757</v>
       </c>
       <c r="D369" s="36" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
     </row>
     <row r="370" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A370" s="35" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B370" t="s">
         <v>141</v>
       </c>
       <c r="C370" s="2" t="s">
-        <v>761</v>
+        <v>757</v>
       </c>
       <c r="D370" s="27"/>
     </row>
     <row r="371" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A371" s="35" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="B371" t="s">
         <v>499</v>
       </c>
       <c r="C371" s="2" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="D371" s="36" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
     </row>
     <row r="372" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A372" s="35" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B372" t="s">
         <v>141</v>
       </c>
       <c r="C372" s="2" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="D372" s="36"/>
     </row>
     <row r="373" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A373" s="35" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="B373" t="s">
         <v>499</v>
       </c>
       <c r="C373" s="2" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="D373" s="36" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
     </row>
     <row r="374" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A374" s="35" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="B374" t="s">
         <v>141</v>
       </c>
       <c r="C374" s="2" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="D374" s="27"/>
     </row>
     <row r="375" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A375" s="35" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="B375" t="s">
         <v>499</v>
       </c>
       <c r="C375" s="2" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="D375" s="36" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
     </row>
     <row r="376" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A376" s="35" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="B376" t="s">
         <v>141</v>
       </c>
       <c r="C376" s="2" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="D376" s="27"/>
     </row>
     <row r="377" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A377" s="35" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="B377" t="s">
         <v>499</v>
       </c>
       <c r="C377" s="2" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="D377" s="36" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
     </row>
     <row r="378" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A378" s="35" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="B378" t="s">
         <v>141</v>
       </c>
       <c r="C378" s="2" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="D378" s="27"/>
     </row>
     <row r="379" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A379" s="35" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="B379" t="s">
         <v>499</v>
       </c>
       <c r="C379" s="2" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="D379" s="36" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
     </row>
     <row r="380" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A380" s="35" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="B380" t="s">
         <v>141</v>
       </c>
       <c r="C380" s="2" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="D380" s="27"/>
     </row>
     <row r="381" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A381" s="35" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="B381" t="s">
         <v>499</v>
       </c>
       <c r="C381" s="2" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="D381" s="36" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
     </row>
     <row r="382" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A382" s="35" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="B382" t="s">
         <v>141</v>
       </c>
       <c r="C382" s="2" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="D382" s="27"/>
     </row>
     <row r="383" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A383" s="35" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="B383" t="s">
         <v>499</v>
       </c>
       <c r="C383" s="2" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="D383" s="36" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
     </row>
     <row r="384" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A384" s="35" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="B384" t="s">
         <v>141</v>
       </c>
       <c r="C384" s="2" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="D384" s="27"/>
     </row>
     <row r="385" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A385" s="35" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="B385" t="s">
         <v>499</v>
       </c>
       <c r="C385" s="2" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="D385" s="36" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
     </row>
     <row r="386" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A386" s="36" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="B386" t="s">
         <v>141</v>
       </c>
       <c r="C386" s="2" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="D386" s="27"/>
     </row>
     <row r="387" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A387" s="36" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="B387" t="s">
         <v>499</v>
       </c>
       <c r="C387" s="2" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="D387" s="27" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
     </row>
     <row r="388" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A388" s="37" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="B388" t="s">
         <v>499</v>
       </c>
       <c r="C388" s="2" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D388" s="27" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
     </row>
     <row r="389" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A389" s="36" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="B389" t="s">
         <v>499</v>
       </c>
       <c r="C389" s="2" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="D389" s="27" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
     </row>
     <row r="390" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A390" s="2" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="B390" t="s">
         <v>499</v>
       </c>
       <c r="C390" s="2" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D390" s="27" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
     </row>
     <row r="391" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A391" s="2" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="B391" t="s">
         <v>499</v>
       </c>
       <c r="C391" s="2" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="D391" s="27" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
     </row>
     <row r="392" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A392" s="2" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="B392" t="s">
         <v>499</v>
       </c>
       <c r="C392" s="2" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="D392" s="27" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
     </row>
     <row r="393" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A393" s="37" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="B393" t="s">
         <v>499</v>
       </c>
       <c r="C393" s="2" t="s">
+        <v>665</v>
+      </c>
+      <c r="D393" s="27" t="s">
         <v>667</v>
-      </c>
-      <c r="D393" s="27" t="s">
-        <v>669</v>
       </c>
     </row>
     <row r="394" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A394" s="37" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="B394" t="s">
         <v>499</v>
       </c>
       <c r="C394" s="2" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="D394" s="27" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
     </row>
     <row r="395" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A395" s="36" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="B395" t="s">
         <v>499</v>
       </c>
       <c r="C395" s="2" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="D395" s="27" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
     </row>
     <row r="396" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A396" s="36" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="B396" t="s">
         <v>499</v>
       </c>
       <c r="C396" s="2" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="D396" s="27" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
     </row>
     <row r="397" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A397" s="2" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="B397" t="s">
         <v>499</v>
       </c>
       <c r="C397" s="2" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="D397" s="27" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
     </row>
     <row r="398" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A398" s="2" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="B398" t="s">
         <v>499</v>
       </c>
       <c r="C398" s="2" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="D398" s="27" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
     </row>
     <row r="399" spans="1:4" x14ac:dyDescent="0.25">
@@ -7753,31 +7913,31 @@
     </row>
     <row r="400" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A400" s="2" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="B400" t="s">
         <v>140</v>
       </c>
       <c r="C400" s="2"/>
       <c r="D400" s="26" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="401" spans="1:4" ht="99" x14ac:dyDescent="0.25">
       <c r="A401" s="2" t="s">
-        <v>739</v>
+        <v>735</v>
       </c>
       <c r="B401" t="s">
         <v>140</v>
       </c>
       <c r="C401" s="2"/>
       <c r="D401" s="40" t="s">
-        <v>775</v>
+        <v>771</v>
       </c>
     </row>
     <row r="402" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A402" s="2" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="B402" t="s">
         <v>141</v>
@@ -7787,21 +7947,21 @@
     </row>
     <row r="403" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A403" s="2" t="s">
-        <v>740</v>
+        <v>736</v>
       </c>
       <c r="B403" t="s">
         <v>140</v>
       </c>
       <c r="C403" s="2" t="s">
-        <v>741</v>
+        <v>737</v>
       </c>
       <c r="D403" s="27" t="s">
-        <v>742</v>
+        <v>738</v>
       </c>
     </row>
     <row r="404" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A404" s="2" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="B404" t="s">
         <v>141</v>
@@ -7811,392 +7971,392 @@
     </row>
     <row r="405" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A405" s="2" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="B405" t="s">
         <v>302</v>
       </c>
       <c r="C405" s="2" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="D405" s="27"/>
     </row>
     <row r="406" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A406" s="2" t="s">
-        <v>699</v>
+        <v>695</v>
       </c>
       <c r="B406" t="s">
         <v>302</v>
       </c>
       <c r="C406" s="2" t="s">
-        <v>701</v>
+        <v>697</v>
       </c>
       <c r="D406" s="27"/>
     </row>
     <row r="407" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A407" s="2" t="s">
-        <v>700</v>
+        <v>696</v>
       </c>
       <c r="B407" t="s">
         <v>302</v>
       </c>
       <c r="C407" s="2" t="s">
-        <v>702</v>
+        <v>698</v>
       </c>
       <c r="D407" s="27"/>
     </row>
     <row r="408" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A408" s="2" t="s">
-        <v>697</v>
+        <v>693</v>
       </c>
       <c r="B408" t="s">
         <v>302</v>
       </c>
       <c r="C408" s="2" t="s">
-        <v>698</v>
+        <v>694</v>
       </c>
       <c r="D408" s="27"/>
     </row>
     <row r="409" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A409" s="2" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="B409" t="s">
         <v>302</v>
       </c>
       <c r="C409" s="2" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="D409" s="27"/>
     </row>
     <row r="410" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A410" s="2" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="B410" t="s">
         <v>302</v>
       </c>
       <c r="C410" s="2" t="s">
-        <v>696</v>
+        <v>692</v>
       </c>
       <c r="D410" s="27"/>
     </row>
     <row r="411" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A411" s="2" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="B411" t="s">
         <v>302</v>
       </c>
       <c r="C411" s="2" t="s">
-        <v>694</v>
+        <v>947</v>
       </c>
       <c r="D411" s="27"/>
     </row>
     <row r="412" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A412" s="2" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="B412" t="s">
         <v>302</v>
       </c>
       <c r="C412" s="2" t="s">
-        <v>695</v>
+        <v>947</v>
       </c>
       <c r="D412" s="27"/>
     </row>
     <row r="413" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A413" s="2" t="s">
-        <v>718</v>
+        <v>714</v>
       </c>
       <c r="B413" t="s">
         <v>140</v>
       </c>
       <c r="C413" s="2"/>
       <c r="D413" s="26" t="s">
-        <v>719</v>
+        <v>715</v>
       </c>
     </row>
     <row r="414" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A414" s="2" t="s">
-        <v>717</v>
+        <v>713</v>
       </c>
       <c r="B414" t="s">
         <v>140</v>
       </c>
       <c r="C414" s="2"/>
       <c r="D414" s="26" t="s">
-        <v>720</v>
+        <v>716</v>
       </c>
     </row>
     <row r="415" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A415" s="2" t="s">
-        <v>723</v>
+        <v>719</v>
       </c>
       <c r="B415" t="s">
         <v>140</v>
       </c>
       <c r="C415" s="2"/>
       <c r="D415" s="38" t="s">
-        <v>722</v>
+        <v>718</v>
       </c>
     </row>
     <row r="416" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A416" s="2" t="s">
-        <v>724</v>
+        <v>720</v>
       </c>
       <c r="B416" t="s">
         <v>140</v>
       </c>
       <c r="C416" s="2" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="D416" s="39" t="s">
-        <v>731</v>
+        <v>727</v>
       </c>
     </row>
     <row r="417" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A417" s="2" t="s">
-        <v>743</v>
+        <v>739</v>
       </c>
       <c r="B417" t="s">
         <v>140</v>
       </c>
       <c r="C417" s="2" t="s">
-        <v>701</v>
+        <v>697</v>
       </c>
       <c r="D417" s="39" t="s">
-        <v>732</v>
+        <v>728</v>
       </c>
     </row>
     <row r="418" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A418" s="2" t="s">
-        <v>725</v>
+        <v>721</v>
       </c>
       <c r="B418" t="s">
         <v>140</v>
       </c>
       <c r="C418" s="2" t="s">
-        <v>702</v>
+        <v>698</v>
       </c>
       <c r="D418" s="39" t="s">
-        <v>733</v>
+        <v>729</v>
       </c>
     </row>
     <row r="419" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A419" s="2" t="s">
-        <v>726</v>
+        <v>722</v>
       </c>
       <c r="B419" t="s">
         <v>140</v>
       </c>
       <c r="C419" s="2" t="s">
-        <v>698</v>
+        <v>694</v>
       </c>
       <c r="D419" s="39" t="s">
-        <v>734</v>
+        <v>730</v>
       </c>
     </row>
     <row r="420" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A420" s="2" t="s">
-        <v>727</v>
+        <v>723</v>
       </c>
       <c r="B420" t="s">
         <v>140</v>
       </c>
       <c r="C420" s="2" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="D420" s="39" t="s">
-        <v>735</v>
+        <v>731</v>
       </c>
     </row>
     <row r="421" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A421" s="2" t="s">
-        <v>728</v>
+        <v>724</v>
       </c>
       <c r="B421" t="s">
         <v>140</v>
       </c>
       <c r="C421" s="2" t="s">
-        <v>696</v>
+        <v>692</v>
       </c>
       <c r="D421" s="39" t="s">
-        <v>736</v>
+        <v>732</v>
       </c>
     </row>
     <row r="422" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A422" s="2" t="s">
-        <v>729</v>
+        <v>725</v>
       </c>
       <c r="B422" t="s">
         <v>140</v>
       </c>
       <c r="C422" s="2" t="s">
-        <v>694</v>
+        <v>947</v>
       </c>
       <c r="D422" s="39" t="s">
-        <v>737</v>
+        <v>733</v>
       </c>
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A423" s="2" t="s">
-        <v>730</v>
+        <v>726</v>
       </c>
       <c r="B423" t="s">
         <v>140</v>
       </c>
       <c r="C423" s="2" t="s">
-        <v>695</v>
+        <v>947</v>
       </c>
       <c r="D423" s="39" t="s">
-        <v>738</v>
+        <v>734</v>
       </c>
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A424" s="2" t="s">
-        <v>721</v>
+        <v>717</v>
       </c>
       <c r="B424" t="s">
         <v>140</v>
       </c>
       <c r="C424" s="2"/>
       <c r="D424" s="38" t="s">
-        <v>711</v>
+        <v>707</v>
       </c>
     </row>
     <row r="425" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A425" s="2" t="s">
-        <v>703</v>
+        <v>699</v>
       </c>
       <c r="B425" t="s">
         <v>140</v>
       </c>
       <c r="C425" s="2" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="D425" s="2" t="s">
-        <v>711</v>
+        <v>707</v>
       </c>
     </row>
     <row r="426" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A426" s="2" t="s">
-        <v>705</v>
+        <v>701</v>
       </c>
       <c r="B426" t="s">
         <v>140</v>
       </c>
       <c r="C426" s="2" t="s">
-        <v>701</v>
+        <v>697</v>
       </c>
       <c r="D426" s="2" t="s">
-        <v>712</v>
+        <v>708</v>
       </c>
     </row>
     <row r="427" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A427" s="2" t="s">
-        <v>706</v>
+        <v>702</v>
       </c>
       <c r="B427" t="s">
         <v>140</v>
       </c>
       <c r="C427" s="2" t="s">
-        <v>702</v>
+        <v>698</v>
       </c>
       <c r="D427" s="2" t="s">
-        <v>713</v>
+        <v>709</v>
       </c>
     </row>
     <row r="428" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A428" s="2" t="s">
-        <v>707</v>
+        <v>703</v>
       </c>
       <c r="B428" t="s">
         <v>140</v>
       </c>
       <c r="C428" s="2" t="s">
-        <v>698</v>
+        <v>694</v>
       </c>
       <c r="D428" s="2" t="s">
-        <v>712</v>
+        <v>708</v>
       </c>
     </row>
     <row r="429" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A429" s="2" t="s">
-        <v>708</v>
+        <v>704</v>
       </c>
       <c r="B429" t="s">
         <v>140</v>
       </c>
       <c r="C429" s="2" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="D429" s="2" t="s">
-        <v>714</v>
+        <v>710</v>
       </c>
     </row>
     <row r="430" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A430" s="2" t="s">
-        <v>704</v>
+        <v>700</v>
       </c>
       <c r="B430" t="s">
         <v>140</v>
       </c>
       <c r="C430" s="2" t="s">
-        <v>696</v>
+        <v>692</v>
       </c>
       <c r="D430" s="2" t="s">
-        <v>714</v>
+        <v>710</v>
       </c>
     </row>
     <row r="431" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A431" s="2" t="s">
-        <v>709</v>
+        <v>705</v>
       </c>
       <c r="B431" t="s">
         <v>140</v>
       </c>
       <c r="C431" s="2" t="s">
-        <v>694</v>
+        <v>947</v>
       </c>
       <c r="D431" s="2" t="s">
-        <v>715</v>
+        <v>711</v>
       </c>
     </row>
     <row r="432" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A432" s="2" t="s">
-        <v>710</v>
+        <v>706</v>
       </c>
       <c r="B432" t="s">
         <v>140</v>
       </c>
       <c r="C432" s="2" t="s">
-        <v>695</v>
+        <v>947</v>
       </c>
       <c r="D432" s="2" t="s">
-        <v>716</v>
+        <v>712</v>
       </c>
     </row>
     <row r="433" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A433" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="B433" t="s">
+        <v>140</v>
+      </c>
+      <c r="D433" s="26" t="s">
         <v>548</v>
-      </c>
-      <c r="B433" t="s">
-        <v>140</v>
-      </c>
-      <c r="D433" s="26" t="s">
-        <v>550</v>
       </c>
     </row>
     <row r="434" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A434" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="B434" t="s">
+        <v>140</v>
+      </c>
+      <c r="D434" s="27" t="s">
         <v>549</v>
-      </c>
-      <c r="B434" t="s">
-        <v>140</v>
-      </c>
-      <c r="D434" s="27" t="s">
-        <v>551</v>
       </c>
     </row>
     <row r="435" spans="1:4" x14ac:dyDescent="0.25">
@@ -8209,13 +8369,13 @@
     </row>
     <row r="436" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A436" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="B436" t="s">
         <v>140</v>
       </c>
       <c r="D436" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
     </row>
     <row r="437" spans="1:4" x14ac:dyDescent="0.25">
@@ -8228,13 +8388,13 @@
     </row>
     <row r="438" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A438" s="2" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="B438" t="s">
         <v>140</v>
       </c>
       <c r="D438" s="33" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
     </row>
     <row r="439" spans="1:4" x14ac:dyDescent="0.25">
@@ -8259,7 +8419,7 @@
         <v>499</v>
       </c>
       <c r="C440" s="2" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="D440" t="s">
         <v>122</v>
@@ -8301,7 +8461,7 @@
         <v>499</v>
       </c>
       <c r="C443" s="2" t="s">
-        <v>516</v>
+        <v>947</v>
       </c>
       <c r="D443" t="s">
         <v>123</v>
@@ -8315,7 +8475,7 @@
         <v>499</v>
       </c>
       <c r="C444" s="2" t="s">
-        <v>517</v>
+        <v>947</v>
       </c>
       <c r="D444" t="s">
         <v>125</v>
@@ -8329,7 +8489,7 @@
         <v>499</v>
       </c>
       <c r="C445" s="2" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D445" t="s">
         <v>124</v>
@@ -8337,111 +8497,111 @@
     </row>
     <row r="446" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A446" s="2" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="B446" t="s">
         <v>140</v>
       </c>
       <c r="C446" s="2"/>
       <c r="D446" s="26" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
     </row>
     <row r="447" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A447" s="2" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="B447" t="s">
         <v>140</v>
       </c>
       <c r="C447" s="2"/>
       <c r="D447" s="10" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
     </row>
     <row r="448" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A448" s="2" t="s">
-        <v>744</v>
+        <v>740</v>
       </c>
       <c r="B448" t="s">
         <v>140</v>
       </c>
       <c r="C448" s="2"/>
       <c r="D448" s="10" t="s">
-        <v>746</v>
+        <v>742</v>
       </c>
     </row>
     <row r="449" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A449" s="2" t="s">
-        <v>745</v>
+        <v>741</v>
       </c>
       <c r="B449" t="s">
         <v>140</v>
       </c>
       <c r="C449" s="2"/>
       <c r="D449" s="10" t="s">
-        <v>747</v>
+        <v>743</v>
       </c>
     </row>
     <row r="450" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A450" s="2" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="B450" t="s">
         <v>140</v>
       </c>
       <c r="C450" s="2" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="D450" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
     </row>
     <row r="451" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A451" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="B451" t="s">
+        <v>140</v>
+      </c>
+      <c r="C451" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="D451" t="s">
         <v>530</v>
-      </c>
-      <c r="B451" t="s">
-        <v>140</v>
-      </c>
-      <c r="C451" s="2" t="s">
-        <v>524</v>
-      </c>
-      <c r="D451" t="s">
-        <v>532</v>
       </c>
     </row>
     <row r="452" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A452" s="30" t="s">
+        <v>535</v>
+      </c>
+      <c r="B452" t="s">
+        <v>140</v>
+      </c>
+      <c r="C452" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="D452" t="s">
         <v>537</v>
-      </c>
-      <c r="B452" t="s">
-        <v>140</v>
-      </c>
-      <c r="C452" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="D452" t="s">
-        <v>539</v>
       </c>
     </row>
     <row r="453" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A453" s="30" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="B453" t="s">
         <v>140</v>
       </c>
       <c r="C453" s="2" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="D453" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
     </row>
     <row r="454" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A454" s="28" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="B454" s="28" t="s">
         <v>141</v>
@@ -8450,7 +8610,7 @@
     </row>
     <row r="455" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A455" s="31" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="B455" s="28" t="s">
         <v>141</v>
@@ -8458,7 +8618,7 @@
     </row>
     <row r="456" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A456" s="28" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B456" s="28" t="s">
         <v>141</v>
@@ -8466,7 +8626,7 @@
     </row>
     <row r="457" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A457" s="32" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="B457" s="28" t="s">
         <v>141</v>
@@ -8474,7 +8634,7 @@
     </row>
     <row r="458" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A458" s="31" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B458" s="28" t="s">
         <v>141</v>
@@ -8482,7 +8642,7 @@
     </row>
     <row r="459" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A459" s="31" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="B459" s="28" t="s">
         <v>141</v>
@@ -8490,7 +8650,7 @@
     </row>
     <row r="460" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A460" s="10" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B460" s="28" t="s">
         <v>141</v>
@@ -8499,7 +8659,7 @@
     </row>
     <row r="461" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A461" s="31" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="B461" s="28" t="s">
         <v>141</v>
@@ -8507,7 +8667,7 @@
     </row>
     <row r="462" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A462" s="32" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="B462" s="28" t="s">
         <v>141</v>
@@ -8516,7 +8676,7 @@
     </row>
     <row r="463" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A463" s="28" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="B463" s="28" t="s">
         <v>141</v>
@@ -8532,7 +8692,7 @@
         <v>510</v>
       </c>
       <c r="C464" s="2" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="465" spans="1:4" x14ac:dyDescent="0.25">
@@ -8543,7 +8703,7 @@
         <v>510</v>
       </c>
       <c r="C465" s="2" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
     </row>
     <row r="466" spans="1:4" x14ac:dyDescent="0.25">
@@ -8554,93 +8714,93 @@
         <v>510</v>
       </c>
       <c r="C466" s="2" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
     </row>
     <row r="467" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A467" s="2" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
       <c r="B467" t="s">
         <v>140</v>
       </c>
       <c r="D467" s="10" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
     </row>
     <row r="468" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A468" s="2" t="s">
-        <v>749</v>
+        <v>745</v>
       </c>
       <c r="B468" t="s">
         <v>140</v>
       </c>
       <c r="C468" t="s">
-        <v>757</v>
+        <v>753</v>
       </c>
       <c r="D468" s="10" t="s">
-        <v>765</v>
+        <v>761</v>
       </c>
     </row>
     <row r="469" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A469" s="2" t="s">
-        <v>750</v>
+        <v>746</v>
       </c>
       <c r="B469" t="s">
         <v>140</v>
       </c>
       <c r="C469" t="s">
-        <v>756</v>
-      </c>
-      <c r="D469" s="41" t="s">
-        <v>766</v>
+        <v>752</v>
+      </c>
+      <c r="D469" t="s">
+        <v>762</v>
       </c>
     </row>
     <row r="470" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A470" s="2" t="s">
-        <v>751</v>
+        <v>747</v>
       </c>
       <c r="B470" t="s">
         <v>140</v>
       </c>
       <c r="C470" t="s">
-        <v>764</v>
+        <v>760</v>
       </c>
       <c r="D470" t="s">
-        <v>767</v>
+        <v>763</v>
       </c>
     </row>
     <row r="471" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A471" s="2" t="s">
-        <v>753</v>
+        <v>749</v>
       </c>
       <c r="B471" t="s">
         <v>140</v>
       </c>
       <c r="C471" t="s">
-        <v>768</v>
+        <v>764</v>
       </c>
       <c r="D471" t="s">
-        <v>769</v>
+        <v>765</v>
       </c>
     </row>
     <row r="472" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A472" s="2" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B472" t="s">
         <v>140</v>
       </c>
       <c r="C472" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="D472" t="s">
-        <v>770</v>
+        <v>766</v>
       </c>
     </row>
     <row r="473" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A473" s="2" t="s">
-        <v>754</v>
+        <v>750</v>
       </c>
       <c r="B473" t="s">
         <v>141</v>
@@ -8648,7 +8808,7 @@
     </row>
     <row r="474" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A474" s="2" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="B474" t="s">
         <v>141</v>
@@ -8656,76 +8816,76 @@
     </row>
     <row r="475" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A475" s="2" t="s">
-        <v>785</v>
+        <v>781</v>
       </c>
       <c r="B475" t="s">
         <v>140</v>
       </c>
-      <c r="C475" s="42" t="s">
-        <v>787</v>
-      </c>
-      <c r="D475" s="43" t="s">
-        <v>787</v>
+      <c r="C475" s="41" t="s">
+        <v>783</v>
+      </c>
+      <c r="D475" s="42" t="s">
+        <v>783</v>
       </c>
     </row>
     <row r="476" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A476" s="2" t="s">
-        <v>786</v>
+        <v>782</v>
       </c>
       <c r="B476" t="s">
         <v>140</v>
       </c>
-      <c r="D476" s="43" t="s">
-        <v>788</v>
+      <c r="D476" s="42" t="s">
+        <v>784</v>
       </c>
     </row>
     <row r="477" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A477" s="2" t="s">
-        <v>789</v>
+        <v>785</v>
       </c>
       <c r="B477" t="s">
         <v>140</v>
       </c>
       <c r="D477" s="38" t="s">
-        <v>791</v>
+        <v>787</v>
       </c>
     </row>
     <row r="478" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A478" s="2" t="s">
-        <v>790</v>
+        <v>786</v>
       </c>
       <c r="B478" t="s">
         <v>140</v>
       </c>
       <c r="D478" t="s">
-        <v>792</v>
+        <v>788</v>
       </c>
     </row>
     <row r="479" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A479" s="2" t="s">
-        <v>795</v>
+        <v>791</v>
       </c>
       <c r="B479" t="s">
         <v>140</v>
       </c>
       <c r="D479" s="38" t="s">
-        <v>793</v>
+        <v>789</v>
       </c>
     </row>
     <row r="480" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A480" s="2" t="s">
-        <v>796</v>
+        <v>792</v>
       </c>
       <c r="B480" t="s">
         <v>140</v>
       </c>
       <c r="D480" t="s">
-        <v>794</v>
+        <v>790</v>
       </c>
     </row>
     <row r="481" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A481" s="2" t="s">
-        <v>797</v>
+        <v>793</v>
       </c>
       <c r="B481" t="s">
         <v>140</v>
@@ -8733,7 +8893,7 @@
     </row>
     <row r="482" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A482" s="2" t="s">
-        <v>798</v>
+        <v>794</v>
       </c>
       <c r="B482" t="s">
         <v>140</v>
@@ -8741,305 +8901,305 @@
     </row>
     <row r="483" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A483" s="2" t="s">
-        <v>773</v>
+        <v>769</v>
       </c>
       <c r="B483" t="s">
         <v>140</v>
       </c>
       <c r="D483" s="10" t="s">
-        <v>774</v>
+        <v>770</v>
       </c>
     </row>
     <row r="484" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A484" s="2" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="B484" t="s">
         <v>140</v>
       </c>
       <c r="C484" t="s">
-        <v>778</v>
-      </c>
-      <c r="D484" s="41" t="s">
-        <v>777</v>
+        <v>774</v>
+      </c>
+      <c r="D484" t="s">
+        <v>773</v>
       </c>
     </row>
     <row r="485" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A485" s="2" t="s">
-        <v>782</v>
+        <v>778</v>
       </c>
       <c r="B485" t="s">
         <v>140</v>
       </c>
       <c r="C485" t="s">
+        <v>775</v>
+      </c>
+      <c r="D485" t="s">
         <v>779</v>
-      </c>
-      <c r="D485" s="41" t="s">
-        <v>783</v>
       </c>
     </row>
     <row r="486" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A486" s="2" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="B486" t="s">
         <v>140</v>
       </c>
       <c r="C486" t="s">
+        <v>776</v>
+      </c>
+      <c r="D486" t="s">
         <v>780</v>
-      </c>
-      <c r="D486" t="s">
-        <v>784</v>
       </c>
     </row>
     <row r="487" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A487" s="2" t="s">
-        <v>799</v>
+        <v>795</v>
       </c>
       <c r="B487" t="s">
         <v>140</v>
       </c>
-      <c r="C487" s="42" t="s">
-        <v>787</v>
-      </c>
-      <c r="D487" s="43" t="s">
-        <v>787</v>
+      <c r="C487" s="41" t="s">
+        <v>783</v>
+      </c>
+      <c r="D487" s="42" t="s">
+        <v>783</v>
       </c>
     </row>
     <row r="488" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A488" s="2" t="s">
-        <v>800</v>
+        <v>796</v>
       </c>
       <c r="B488" t="s">
         <v>140</v>
       </c>
-      <c r="D488" s="43" t="s">
-        <v>788</v>
+      <c r="D488" s="42" t="s">
+        <v>784</v>
       </c>
     </row>
     <row r="489" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A489" s="2" t="s">
-        <v>822</v>
+        <v>818</v>
       </c>
       <c r="B489" t="s">
         <v>140</v>
       </c>
       <c r="D489" s="38" t="s">
-        <v>802</v>
+        <v>798</v>
       </c>
     </row>
     <row r="490" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A490" s="2" t="s">
-        <v>823</v>
+        <v>819</v>
       </c>
       <c r="B490" t="s">
         <v>140</v>
       </c>
-      <c r="D490" s="44" t="s">
-        <v>803</v>
+      <c r="D490" s="43" t="s">
+        <v>799</v>
       </c>
     </row>
     <row r="491" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A491" s="2" t="s">
-        <v>824</v>
+        <v>820</v>
       </c>
       <c r="B491" t="s">
         <v>140</v>
       </c>
       <c r="D491" s="38" t="s">
-        <v>804</v>
+        <v>800</v>
       </c>
     </row>
     <row r="492" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A492" s="2" t="s">
-        <v>825</v>
+        <v>821</v>
       </c>
       <c r="B492" t="s">
         <v>140</v>
       </c>
-      <c r="D492" s="45" t="s">
-        <v>805</v>
+      <c r="D492" s="44" t="s">
+        <v>801</v>
       </c>
     </row>
     <row r="493" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A493" s="2" t="s">
-        <v>826</v>
+        <v>822</v>
       </c>
       <c r="B493" t="s">
         <v>140</v>
       </c>
       <c r="D493" s="38" t="s">
-        <v>806</v>
+        <v>802</v>
       </c>
     </row>
     <row r="494" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A494" s="2" t="s">
-        <v>827</v>
+        <v>823</v>
       </c>
       <c r="B494" t="s">
         <v>140</v>
       </c>
-      <c r="D494" s="45" t="s">
-        <v>807</v>
+      <c r="D494" s="44" t="s">
+        <v>803</v>
       </c>
     </row>
     <row r="495" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A495" s="2" t="s">
-        <v>828</v>
+        <v>824</v>
       </c>
       <c r="B495" t="s">
         <v>140</v>
       </c>
       <c r="D495" s="38" t="s">
-        <v>808</v>
+        <v>804</v>
       </c>
     </row>
     <row r="496" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A496" s="2" t="s">
-        <v>829</v>
+        <v>825</v>
       </c>
       <c r="B496" t="s">
         <v>140</v>
       </c>
-      <c r="D496" s="45" t="s">
-        <v>809</v>
+      <c r="D496" s="44" t="s">
+        <v>805</v>
       </c>
     </row>
     <row r="497" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A497" s="2" t="s">
-        <v>830</v>
+        <v>826</v>
       </c>
       <c r="B497" t="s">
         <v>140</v>
       </c>
       <c r="D497" s="38" t="s">
-        <v>810</v>
+        <v>806</v>
       </c>
     </row>
     <row r="498" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A498" s="2" t="s">
-        <v>831</v>
+        <v>827</v>
       </c>
       <c r="B498" t="s">
         <v>140</v>
       </c>
-      <c r="D498" s="45" t="s">
-        <v>811</v>
+      <c r="D498" s="44" t="s">
+        <v>807</v>
       </c>
     </row>
     <row r="499" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A499" s="2" t="s">
-        <v>832</v>
+        <v>828</v>
       </c>
       <c r="B499" t="s">
         <v>140</v>
       </c>
       <c r="D499" s="39" t="s">
-        <v>812</v>
+        <v>808</v>
       </c>
     </row>
     <row r="500" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A500" s="2" t="s">
-        <v>833</v>
+        <v>829</v>
       </c>
       <c r="B500" t="s">
         <v>140</v>
       </c>
       <c r="D500" s="38" t="s">
-        <v>813</v>
+        <v>809</v>
       </c>
     </row>
     <row r="501" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A501" s="2" t="s">
-        <v>834</v>
+        <v>830</v>
       </c>
       <c r="B501" t="s">
         <v>140</v>
       </c>
       <c r="D501" s="39" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
     </row>
     <row r="502" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A502" s="2" t="s">
-        <v>835</v>
+        <v>831</v>
       </c>
       <c r="B502" t="s">
         <v>140</v>
       </c>
       <c r="D502" s="38" t="s">
-        <v>815</v>
+        <v>811</v>
       </c>
     </row>
     <row r="503" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A503" s="2" t="s">
-        <v>838</v>
+        <v>834</v>
       </c>
       <c r="B503" t="s">
         <v>140</v>
       </c>
       <c r="D503" s="39" t="s">
-        <v>816</v>
+        <v>812</v>
       </c>
     </row>
     <row r="504" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A504" s="2" t="s">
-        <v>839</v>
+        <v>835</v>
       </c>
       <c r="B504" t="s">
         <v>140</v>
       </c>
       <c r="D504" s="38" t="s">
-        <v>817</v>
+        <v>813</v>
       </c>
     </row>
     <row r="505" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A505" s="2" t="s">
-        <v>836</v>
+        <v>832</v>
       </c>
       <c r="B505" t="s">
         <v>140</v>
       </c>
       <c r="D505" s="39" t="s">
-        <v>818</v>
+        <v>814</v>
       </c>
     </row>
     <row r="506" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A506" s="2" t="s">
-        <v>837</v>
+        <v>833</v>
       </c>
       <c r="B506" t="s">
         <v>140</v>
       </c>
       <c r="D506" s="38" t="s">
-        <v>819</v>
+        <v>815</v>
       </c>
     </row>
     <row r="507" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A507" s="2" t="s">
-        <v>840</v>
+        <v>836</v>
       </c>
       <c r="B507" t="s">
         <v>140</v>
       </c>
       <c r="D507" s="39" t="s">
-        <v>820</v>
+        <v>816</v>
       </c>
     </row>
     <row r="508" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A508" s="2" t="s">
-        <v>841</v>
+        <v>837</v>
       </c>
       <c r="B508" t="s">
         <v>140</v>
       </c>
       <c r="D508" s="38" t="s">
-        <v>821</v>
+        <v>817</v>
       </c>
     </row>
     <row r="509" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A509" s="2" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="B509" t="s">
         <v>302</v>
@@ -9047,7 +9207,7 @@
     </row>
     <row r="510" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A510" s="2" t="s">
-        <v>801</v>
+        <v>797</v>
       </c>
       <c r="B510" t="s">
         <v>302</v>
@@ -9055,497 +9215,745 @@
     </row>
     <row r="511" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A511" s="2" t="s">
-        <v>842</v>
+        <v>838</v>
       </c>
       <c r="B511" t="s">
         <v>140</v>
       </c>
-      <c r="D511" s="46" t="s">
-        <v>843</v>
+      <c r="D511" s="45" t="s">
+        <v>839</v>
       </c>
     </row>
     <row r="512" spans="1:4" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A512" s="2" t="s">
-        <v>844</v>
+        <v>840</v>
       </c>
       <c r="B512" t="s">
         <v>140</v>
       </c>
-      <c r="D512" s="47" t="s">
-        <v>845</v>
+      <c r="D512" s="46" t="s">
+        <v>841</v>
       </c>
     </row>
     <row r="513" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A513" s="2" t="s">
-        <v>846</v>
+        <v>842</v>
       </c>
       <c r="B513" t="s">
         <v>140</v>
       </c>
-      <c r="D513" s="43" t="s">
-        <v>849</v>
+      <c r="D513" s="42" t="s">
+        <v>845</v>
       </c>
     </row>
     <row r="514" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A514" s="2" t="s">
-        <v>847</v>
+        <v>843</v>
       </c>
       <c r="B514" t="s">
         <v>140</v>
       </c>
-      <c r="D514" s="43" t="s">
-        <v>850</v>
+      <c r="D514" s="42" t="s">
+        <v>846</v>
       </c>
     </row>
     <row r="515" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A515" s="2" t="s">
-        <v>848</v>
+        <v>844</v>
       </c>
       <c r="B515" t="s">
         <v>140</v>
       </c>
-      <c r="D515" s="43" t="s">
-        <v>851</v>
+      <c r="D515" s="42" t="s">
+        <v>847</v>
       </c>
     </row>
     <row r="516" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A516" s="2" t="s">
-        <v>852</v>
+        <v>848</v>
       </c>
       <c r="B516" t="s">
         <v>140</v>
       </c>
       <c r="D516" s="38" t="s">
-        <v>858</v>
+        <v>854</v>
       </c>
     </row>
     <row r="517" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A517" s="2" t="s">
-        <v>853</v>
+        <v>849</v>
       </c>
       <c r="B517" t="s">
         <v>140</v>
       </c>
       <c r="D517" s="38" t="s">
-        <v>859</v>
+        <v>855</v>
       </c>
     </row>
     <row r="518" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A518" s="2" t="s">
-        <v>854</v>
+        <v>850</v>
       </c>
       <c r="B518" t="s">
         <v>140</v>
       </c>
       <c r="D518" s="38" t="s">
-        <v>863</v>
+        <v>859</v>
       </c>
     </row>
     <row r="519" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A519" s="2" t="s">
-        <v>855</v>
+        <v>851</v>
       </c>
       <c r="B519" t="s">
         <v>140</v>
       </c>
       <c r="D519" s="38" t="s">
-        <v>860</v>
+        <v>856</v>
       </c>
     </row>
     <row r="520" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A520" s="2" t="s">
-        <v>856</v>
+        <v>852</v>
       </c>
       <c r="B520" t="s">
         <v>140</v>
       </c>
       <c r="D520" s="38" t="s">
-        <v>861</v>
+        <v>857</v>
       </c>
     </row>
     <row r="521" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A521" s="2" t="s">
-        <v>857</v>
+        <v>853</v>
       </c>
       <c r="B521" t="s">
         <v>140</v>
       </c>
       <c r="D521" s="38" t="s">
-        <v>862</v>
+        <v>858</v>
       </c>
     </row>
     <row r="522" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A522" s="2" t="s">
-        <v>864</v>
+        <v>860</v>
       </c>
       <c r="B522" t="s">
         <v>140</v>
       </c>
       <c r="D522" s="38" t="s">
-        <v>870</v>
+        <v>866</v>
       </c>
     </row>
     <row r="523" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A523" s="2" t="s">
-        <v>865</v>
+        <v>861</v>
       </c>
       <c r="B523" t="s">
         <v>140</v>
       </c>
       <c r="D523" s="38" t="s">
-        <v>871</v>
+        <v>867</v>
       </c>
     </row>
     <row r="524" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A524" s="2" t="s">
-        <v>866</v>
+        <v>862</v>
       </c>
       <c r="B524" t="s">
         <v>140</v>
       </c>
       <c r="D524" s="38" t="s">
-        <v>872</v>
+        <v>868</v>
       </c>
     </row>
     <row r="525" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A525" s="2" t="s">
-        <v>867</v>
+        <v>863</v>
       </c>
       <c r="B525" t="s">
         <v>140</v>
       </c>
       <c r="D525" s="38" t="s">
-        <v>873</v>
+        <v>869</v>
       </c>
     </row>
     <row r="526" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A526" s="2" t="s">
-        <v>868</v>
+        <v>864</v>
       </c>
       <c r="B526" t="s">
         <v>140</v>
       </c>
       <c r="D526" s="38" t="s">
-        <v>874</v>
+        <v>870</v>
       </c>
     </row>
     <row r="527" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A527" s="2" t="s">
-        <v>869</v>
+        <v>865</v>
       </c>
       <c r="B527" t="s">
         <v>140</v>
       </c>
       <c r="D527" s="38" t="s">
-        <v>875</v>
+        <v>871</v>
       </c>
     </row>
     <row r="528" spans="1:4" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A528" s="2" t="s">
-        <v>882</v>
+        <v>878</v>
       </c>
       <c r="B528" t="s">
         <v>140</v>
       </c>
-      <c r="D528" s="48" t="s">
-        <v>876</v>
+      <c r="D528" s="47" t="s">
+        <v>872</v>
       </c>
     </row>
     <row r="529" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A529" s="2" t="s">
-        <v>883</v>
+        <v>879</v>
       </c>
       <c r="B529" t="s">
         <v>140</v>
       </c>
-      <c r="D529" s="49" t="s">
-        <v>877</v>
+      <c r="D529" s="48" t="s">
+        <v>873</v>
       </c>
     </row>
     <row r="530" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A530" s="2" t="s">
-        <v>884</v>
+        <v>880</v>
       </c>
       <c r="B530" t="s">
         <v>140</v>
       </c>
-      <c r="D530" s="49" t="s">
-        <v>878</v>
+      <c r="D530" s="48" t="s">
+        <v>874</v>
       </c>
     </row>
     <row r="531" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A531" s="2" t="s">
-        <v>885</v>
+        <v>881</v>
       </c>
       <c r="B531" t="s">
         <v>140</v>
       </c>
-      <c r="D531" s="49" t="s">
-        <v>879</v>
+      <c r="D531" s="48" t="s">
+        <v>875</v>
       </c>
     </row>
     <row r="532" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A532" s="2" t="s">
-        <v>886</v>
+        <v>882</v>
       </c>
       <c r="B532" t="s">
         <v>140</v>
       </c>
-      <c r="D532" s="49" t="s">
-        <v>880</v>
+      <c r="D532" s="48" t="s">
+        <v>876</v>
       </c>
     </row>
     <row r="533" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A533" s="2" t="s">
-        <v>887</v>
+        <v>883</v>
       </c>
       <c r="B533" t="s">
         <v>140</v>
       </c>
-      <c r="D533" s="49" t="s">
-        <v>881</v>
+      <c r="D533" s="48" t="s">
+        <v>877</v>
       </c>
     </row>
     <row r="534" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A534" s="2" t="s">
-        <v>888</v>
+        <v>884</v>
       </c>
       <c r="B534" t="s">
         <v>140</v>
       </c>
       <c r="D534" s="10" t="s">
-        <v>889</v>
+        <v>885</v>
       </c>
     </row>
     <row r="535" spans="1:4" ht="210" x14ac:dyDescent="0.25">
       <c r="A535" s="2" t="s">
-        <v>891</v>
+        <v>887</v>
       </c>
       <c r="B535" t="s">
         <v>140</v>
       </c>
       <c r="D535" s="13" t="s">
-        <v>890</v>
+        <v>886</v>
       </c>
     </row>
     <row r="536" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A536" s="2" t="s">
-        <v>892</v>
+        <v>888</v>
       </c>
       <c r="B536" t="s">
         <v>140</v>
       </c>
-      <c r="D536" s="46" t="s">
-        <v>893</v>
+      <c r="D536" s="45" t="s">
+        <v>889</v>
       </c>
     </row>
     <row r="537" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A537" s="2" t="s">
-        <v>894</v>
+        <v>890</v>
       </c>
       <c r="B537" t="s">
         <v>140</v>
       </c>
       <c r="D537" s="27" t="s">
-        <v>895</v>
+        <v>891</v>
       </c>
     </row>
     <row r="538" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A538" s="2" t="s">
-        <v>900</v>
+        <v>896</v>
       </c>
       <c r="B538" t="s">
         <v>140</v>
       </c>
-      <c r="D538" s="43" t="s">
-        <v>896</v>
+      <c r="D538" s="42" t="s">
+        <v>892</v>
       </c>
     </row>
     <row r="539" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A539" s="2" t="s">
-        <v>901</v>
+        <v>897</v>
       </c>
       <c r="B539" t="s">
         <v>140</v>
       </c>
-      <c r="D539" s="43" t="s">
-        <v>850</v>
+      <c r="D539" s="42" t="s">
+        <v>846</v>
       </c>
     </row>
     <row r="540" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A540" s="2" t="s">
-        <v>902</v>
+        <v>898</v>
       </c>
       <c r="B540" t="s">
         <v>140</v>
       </c>
       <c r="D540" t="s">
-        <v>897</v>
+        <v>893</v>
       </c>
     </row>
     <row r="541" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A541" s="2" t="s">
-        <v>898</v>
+        <v>894</v>
       </c>
       <c r="B541" t="s">
         <v>140</v>
       </c>
-      <c r="D541" s="50" t="s">
+      <c r="D541" s="49" t="s">
         <v>390</v>
       </c>
     </row>
     <row r="542" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A542" s="2" t="s">
-        <v>899</v>
+        <v>895</v>
       </c>
       <c r="B542" t="s">
         <v>140</v>
       </c>
-      <c r="D542" s="51" t="s">
+      <c r="D542" s="50" t="s">
         <v>411</v>
       </c>
     </row>
     <row r="543" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A543" s="2" t="s">
-        <v>903</v>
+        <v>899</v>
       </c>
       <c r="B543" t="s">
         <v>140</v>
       </c>
-      <c r="D543" s="51" t="s">
+      <c r="D543" s="50" t="s">
         <v>408</v>
       </c>
     </row>
     <row r="544" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A544" s="2" t="s">
-        <v>904</v>
+        <v>900</v>
       </c>
       <c r="B544" t="s">
         <v>140</v>
       </c>
-      <c r="D544" s="51" t="s">
+      <c r="D544" s="50" t="s">
         <v>399</v>
       </c>
     </row>
     <row r="545" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A545" s="2" t="s">
-        <v>905</v>
+        <v>901</v>
       </c>
       <c r="B545" t="s">
         <v>140</v>
       </c>
-      <c r="D545" s="51" t="s">
-        <v>906</v>
+      <c r="D545" s="50" t="s">
+        <v>902</v>
       </c>
     </row>
     <row r="546" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A546" s="2" t="s">
-        <v>915</v>
+        <v>911</v>
       </c>
       <c r="B546" t="s">
         <v>140</v>
       </c>
-      <c r="D546" s="50" t="s">
-        <v>907</v>
+      <c r="D546" s="49" t="s">
+        <v>903</v>
       </c>
     </row>
     <row r="547" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A547" s="2" t="s">
-        <v>916</v>
+        <v>912</v>
       </c>
       <c r="B547" t="s">
         <v>140</v>
       </c>
-      <c r="D547" s="51" t="s">
-        <v>874</v>
+      <c r="D547" s="50" t="s">
+        <v>870</v>
       </c>
     </row>
     <row r="548" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A548" s="2" t="s">
-        <v>917</v>
+        <v>913</v>
       </c>
       <c r="B548" t="s">
         <v>140</v>
       </c>
-      <c r="D548" s="51" t="s">
-        <v>908</v>
+      <c r="D548" s="50" t="s">
+        <v>904</v>
       </c>
     </row>
     <row r="549" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A549" s="2" t="s">
-        <v>918</v>
+        <v>914</v>
       </c>
       <c r="B549" t="s">
         <v>140</v>
       </c>
-      <c r="D549" s="51" t="s">
-        <v>871</v>
+      <c r="D549" s="50" t="s">
+        <v>867</v>
       </c>
     </row>
     <row r="550" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A550" s="2" t="s">
-        <v>919</v>
+        <v>915</v>
       </c>
       <c r="B550" t="s">
         <v>140</v>
       </c>
-      <c r="D550" s="51" t="s">
-        <v>909</v>
+      <c r="D550" s="50" t="s">
+        <v>905</v>
       </c>
     </row>
     <row r="551" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A551" s="2" t="s">
-        <v>920</v>
+        <v>916</v>
       </c>
       <c r="B551" t="s">
         <v>140</v>
       </c>
-      <c r="D551" s="50" t="s">
-        <v>910</v>
+      <c r="D551" s="49" t="s">
+        <v>906</v>
       </c>
     </row>
     <row r="552" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A552" s="2" t="s">
-        <v>921</v>
+        <v>917</v>
       </c>
       <c r="B552" t="s">
         <v>140</v>
       </c>
-      <c r="D552" s="51" t="s">
-        <v>911</v>
+      <c r="D552" s="50" t="s">
+        <v>907</v>
       </c>
     </row>
     <row r="553" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A553" s="2" t="s">
-        <v>922</v>
+        <v>918</v>
       </c>
       <c r="B553" t="s">
         <v>140</v>
       </c>
-      <c r="D553" s="51" t="s">
-        <v>912</v>
+      <c r="D553" s="50" t="s">
+        <v>908</v>
       </c>
     </row>
     <row r="554" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A554" s="2" t="s">
-        <v>923</v>
+        <v>919</v>
       </c>
       <c r="B554" t="s">
         <v>140</v>
       </c>
-      <c r="D554" s="51" t="s">
-        <v>913</v>
+      <c r="D554" s="50" t="s">
+        <v>909</v>
       </c>
     </row>
     <row r="555" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A555" s="2" t="s">
-        <v>924</v>
+        <v>920</v>
       </c>
       <c r="B555" t="s">
         <v>140</v>
       </c>
-      <c r="D555" s="51" t="s">
-        <v>914</v>
+      <c r="D555" s="50" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="556" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A556" s="2" t="s">
+        <v>940</v>
+      </c>
+      <c r="B556" t="s">
+        <v>140</v>
+      </c>
+      <c r="D556" s="10" t="s">
+        <v>938</v>
+      </c>
+    </row>
+    <row r="557" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A557" s="2" t="s">
+        <v>941</v>
+      </c>
+      <c r="B557" t="s">
+        <v>140</v>
+      </c>
+      <c r="D557" s="51" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="558" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A558" s="2" t="s">
+        <v>934</v>
+      </c>
+      <c r="B558" t="s">
+        <v>140</v>
+      </c>
+      <c r="C558" s="2" t="s">
+        <v>947</v>
+      </c>
+      <c r="D558" s="27" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="559" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A559" s="2" t="s">
+        <v>936</v>
+      </c>
+      <c r="B559" t="s">
+        <v>140</v>
+      </c>
+      <c r="D559" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="560" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A560" s="2" t="s">
+        <v>942</v>
+      </c>
+      <c r="B560" t="s">
+        <v>140</v>
+      </c>
+      <c r="D560" s="10" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="561" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A561" s="2" t="s">
+        <v>944</v>
+      </c>
+      <c r="B561" t="s">
+        <v>140</v>
+      </c>
+      <c r="D561" t="s">
+        <v>946</v>
+      </c>
+    </row>
+    <row r="562" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A562" s="28" t="s">
+        <v>945</v>
+      </c>
+      <c r="B562" s="29" t="s">
+        <v>510</v>
+      </c>
+      <c r="C562" s="29"/>
+    </row>
+    <row r="563" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A563" s="2" t="s">
+        <v>932</v>
+      </c>
+      <c r="B563" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="564" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A564" s="2" t="s">
+        <v>933</v>
+      </c>
+      <c r="B564" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="565" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A565" s="2" t="s">
+        <v>950</v>
+      </c>
+      <c r="D565" s="26" t="s">
+        <v>949</v>
+      </c>
+    </row>
+    <row r="566" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A566" s="2" t="s">
+        <v>952</v>
+      </c>
+      <c r="D566" s="10" t="s">
+        <v>948</v>
+      </c>
+    </row>
+    <row r="567" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A567" s="2" t="s">
+        <v>951</v>
+      </c>
+    </row>
+    <row r="568" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A568" s="2" t="s">
+        <v>953</v>
+      </c>
+    </row>
+    <row r="569" spans="1:4" ht="33" x14ac:dyDescent="0.3">
+      <c r="A569" s="10" t="s">
+        <v>960</v>
+      </c>
+      <c r="D569" s="52" t="s">
+        <v>959</v>
+      </c>
+    </row>
+    <row r="570" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A570" s="30" t="s">
+        <v>954</v>
+      </c>
+      <c r="D570" t="s">
+        <v>961</v>
+      </c>
+    </row>
+    <row r="571" spans="1:4" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="A571" s="10" t="s">
+        <v>962</v>
+      </c>
+      <c r="D571" s="52" t="s">
+        <v>963</v>
+      </c>
+    </row>
+    <row r="572" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A572" s="10" t="s">
+        <v>965</v>
+      </c>
+      <c r="D572" s="10" t="s">
+        <v>966</v>
+      </c>
+    </row>
+    <row r="573" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A573" s="10" t="s">
+        <v>964</v>
+      </c>
+      <c r="D573" s="10" t="s">
+        <v>967</v>
+      </c>
+    </row>
+    <row r="574" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A574" s="10" t="s">
+        <v>968</v>
+      </c>
+      <c r="D574" s="10" t="s">
+        <v>969</v>
+      </c>
+    </row>
+    <row r="575" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A575" s="10" t="s">
+        <v>970</v>
+      </c>
+      <c r="D575" s="10" t="s">
+        <v>971</v>
+      </c>
+    </row>
+    <row r="576" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A576" s="10" t="s">
+        <v>972</v>
+      </c>
+      <c r="D576" s="10" t="s">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="577" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A577" s="10" t="s">
+        <v>974</v>
+      </c>
+      <c r="D577" s="10" t="s">
+        <v>975</v>
+      </c>
+    </row>
+    <row r="578" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A578" s="10" t="s">
+        <v>976</v>
+      </c>
+      <c r="D578" s="10" t="s">
+        <v>977</v>
+      </c>
+    </row>
+    <row r="579" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A579" s="10" t="s">
+        <v>978</v>
+      </c>
+      <c r="D579" s="10" t="s">
+        <v>979</v>
+      </c>
+    </row>
+    <row r="580" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A580" s="10" t="s">
+        <v>980</v>
+      </c>
+      <c r="D580" s="10" t="s">
+        <v>981</v>
+      </c>
+    </row>
+    <row r="581" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A581" s="10" t="s">
+        <v>982</v>
+      </c>
+      <c r="D581" s="10" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="582" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A582" s="10" t="s">
+        <v>984</v>
+      </c>
+      <c r="D582" s="10" t="s">
+        <v>985</v>
+      </c>
+    </row>
+    <row r="590" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A590" s="2" t="s">
+        <v>956</v>
+      </c>
+      <c r="D590" s="10" t="s">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="591" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A591" s="2" t="s">
+        <v>958</v>
+      </c>
+      <c r="D591" s="10" t="s">
+        <v>957</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update resource templates and references
Replace updated binary resource files in inst/resources: protocol_schema_iphra.xlsx, reach_tor_iphra_template.docx, and reference.xlsx. These refresh the package's schema, TOR template, and reference spreadsheets; no source code changes were made.
</commit_message>
<xml_diff>
--- a/inst/resources/protocol_schema_iphra.xlsx
+++ b/inst/resources/protocol_schema_iphra.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R Projects\SaeedR1987\public_health_resources\inst\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{835BF67D-99B0-49B8-99A6-0DE7E5559656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF664CA5-BA30-46ED-829B-80A324E80FC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-14505" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="schema" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1618" uniqueCount="986">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1652" uniqueCount="991">
   <si>
     <t>tag_name</t>
   </si>
@@ -3129,9 +3129,6 @@
     <t>Data will be collected using a contextualized IPHRA ODK tool. Cleaning and analysis will be done using a pre-prepared IPHRA application built in @r_version.</t>
   </si>
   <si>
-    <t>@text_intro_data_processing_analysis</t>
-  </si>
-  <si>
     <t>The household analysis will be treated as a simple random sampling design across sites without applying survey weights. @text_analysis_fpc_unstratified.</t>
   </si>
   <si>
@@ -3205,6 +3202,24 @@
   </si>
   <si>
     <t>The ratio of children 0-23 months of age to children 24-59 months of age in the sample will be evaluated to determine if additional age weighting is needed for analysis of the indicator Global or Severe Acute Malnutrition by MUAC. If strong differences are observed against an expected proportion of two-thirds children 24-59 months out of all under-5 year old children, then a set of weights will be applied if the child is 0-23 months or 24-59 months for this specific indicator. The age weights will be multiplied with any household level weights to generate a single set of composite weight for analysis.</t>
+  </si>
+  <si>
+    <t>@text_intro_household_survey_analysis</t>
+  </si>
+  <si>
+    <t>muac_survey</t>
+  </si>
+  <si>
+    <t>@header_analysis_kii_obs</t>
+  </si>
+  <si>
+    <t>Key Informant Interview and Observation Data</t>
+  </si>
+  <si>
+    <t>@text_analysis_kii_obs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Community key informant interviews and community observation checklists will be qualitatively analysed using a data saturation grid, with the objectives of (a) triangulating the self-perceived needs of the population against quantitative data, and (b) attaining a better qualitative understanding of the nature of needs and barriers. The qualitative analysis uses a two-step process: Firstly, qualitative responses or observations are categorized as pertaining to one or more pillars or sub-pillars of the Acute Needs Framework to facilitate comparison of results across tools; and secondly a rapid coding is conducted to identify common themes and issues within pillars. Responses will be compared across gender and assessed sites. A standardized data saturation grid is used to facilitate this analysis. </t>
   </si>
 </sst>
 </file>
@@ -3465,7 +3480,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -3555,7 +3570,6 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
@@ -3861,7 +3875,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D591"/>
+  <dimension ref="A1:D586"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="53.140625" customWidth="1"/>
@@ -9726,7 +9740,7 @@
       <c r="B557" t="s">
         <v>140</v>
       </c>
-      <c r="D557" s="51" t="s">
+      <c r="D557" t="s">
         <v>939</v>
       </c>
     </row>
@@ -9751,6 +9765,9 @@
       <c r="B559" t="s">
         <v>140</v>
       </c>
+      <c r="C559" t="s">
+        <v>986</v>
+      </c>
       <c r="D559" t="s">
         <v>937</v>
       </c>
@@ -9806,6 +9823,9 @@
       <c r="A565" s="2" t="s">
         <v>950</v>
       </c>
+      <c r="B565" t="s">
+        <v>140</v>
+      </c>
       <c r="D565" s="26" t="s">
         <v>949</v>
       </c>
@@ -9814,6 +9834,9 @@
       <c r="A566" s="2" t="s">
         <v>952</v>
       </c>
+      <c r="B566" t="s">
+        <v>140</v>
+      </c>
       <c r="D566" s="10" t="s">
         <v>948</v>
       </c>
@@ -9822,17 +9845,26 @@
       <c r="A567" s="2" t="s">
         <v>951</v>
       </c>
+      <c r="B567" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="568" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A568" s="2" t="s">
         <v>953</v>
       </c>
+      <c r="B568" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="569" spans="1:4" ht="33" x14ac:dyDescent="0.3">
-      <c r="A569" s="10" t="s">
-        <v>960</v>
-      </c>
-      <c r="D569" s="52" t="s">
+      <c r="A569" s="30" t="s">
+        <v>985</v>
+      </c>
+      <c r="B569" t="s">
+        <v>140</v>
+      </c>
+      <c r="D569" s="51" t="s">
         <v>959</v>
       </c>
     </row>
@@ -9840,120 +9872,208 @@
       <c r="A570" s="30" t="s">
         <v>954</v>
       </c>
+      <c r="B570" t="s">
+        <v>140</v>
+      </c>
       <c r="D570" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
     </row>
     <row r="571" spans="1:4" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A571" s="10" t="s">
+        <v>961</v>
+      </c>
+      <c r="B571" t="s">
+        <v>140</v>
+      </c>
+      <c r="C571" s="2" t="s">
+        <v>737</v>
+      </c>
+      <c r="D571" s="51" t="s">
         <v>962</v>
-      </c>
-      <c r="D571" s="52" t="s">
-        <v>963</v>
       </c>
     </row>
     <row r="572" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A572" s="10" t="s">
+        <v>964</v>
+      </c>
+      <c r="B572" t="s">
+        <v>140</v>
+      </c>
+      <c r="D572" s="10" t="s">
         <v>965</v>
-      </c>
-      <c r="D572" s="10" t="s">
-        <v>966</v>
       </c>
     </row>
     <row r="573" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A573" s="10" t="s">
-        <v>964</v>
+        <v>963</v>
+      </c>
+      <c r="B573" t="s">
+        <v>140</v>
+      </c>
+      <c r="C573" s="2" t="s">
+        <v>737</v>
       </c>
       <c r="D573" s="10" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
     </row>
     <row r="574" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A574" s="10" t="s">
+        <v>967</v>
+      </c>
+      <c r="B574" t="s">
+        <v>140</v>
+      </c>
+      <c r="D574" s="10" t="s">
         <v>968</v>
-      </c>
-      <c r="D574" s="10" t="s">
-        <v>969</v>
       </c>
     </row>
     <row r="575" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A575" s="10" t="s">
+        <v>969</v>
+      </c>
+      <c r="B575" t="s">
+        <v>140</v>
+      </c>
+      <c r="C575" s="2" t="s">
+        <v>737</v>
+      </c>
+      <c r="D575" s="10" t="s">
         <v>970</v>
-      </c>
-      <c r="D575" s="10" t="s">
-        <v>971</v>
       </c>
     </row>
     <row r="576" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A576" s="10" t="s">
+        <v>971</v>
+      </c>
+      <c r="B576" t="s">
+        <v>140</v>
+      </c>
+      <c r="D576" s="10" t="s">
         <v>972</v>
-      </c>
-      <c r="D576" s="10" t="s">
-        <v>973</v>
       </c>
     </row>
     <row r="577" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A577" s="10" t="s">
+        <v>973</v>
+      </c>
+      <c r="B577" t="s">
+        <v>140</v>
+      </c>
+      <c r="C577" s="2" t="s">
+        <v>737</v>
+      </c>
+      <c r="D577" s="10" t="s">
         <v>974</v>
-      </c>
-      <c r="D577" s="10" t="s">
-        <v>975</v>
       </c>
     </row>
     <row r="578" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A578" s="10" t="s">
+        <v>975</v>
+      </c>
+      <c r="B578" t="s">
+        <v>140</v>
+      </c>
+      <c r="D578" s="10" t="s">
         <v>976</v>
-      </c>
-      <c r="D578" s="10" t="s">
-        <v>977</v>
       </c>
     </row>
     <row r="579" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A579" s="10" t="s">
+        <v>977</v>
+      </c>
+      <c r="B579" t="s">
+        <v>140</v>
+      </c>
+      <c r="C579" s="2" t="s">
+        <v>737</v>
+      </c>
+      <c r="D579" s="10" t="s">
         <v>978</v>
-      </c>
-      <c r="D579" s="10" t="s">
-        <v>979</v>
       </c>
     </row>
     <row r="580" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A580" s="10" t="s">
+        <v>979</v>
+      </c>
+      <c r="B580" t="s">
+        <v>140</v>
+      </c>
+      <c r="D580" s="10" t="s">
         <v>980</v>
-      </c>
-      <c r="D580" s="10" t="s">
-        <v>981</v>
       </c>
     </row>
     <row r="581" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A581" s="10" t="s">
+        <v>981</v>
+      </c>
+      <c r="B581" t="s">
+        <v>140</v>
+      </c>
+      <c r="C581" s="2" t="s">
+        <v>737</v>
+      </c>
+      <c r="D581" s="10" t="s">
         <v>982</v>
-      </c>
-      <c r="D581" s="10" t="s">
-        <v>983</v>
       </c>
     </row>
     <row r="582" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A582" s="10" t="s">
+        <v>983</v>
+      </c>
+      <c r="B582" t="s">
+        <v>140</v>
+      </c>
+      <c r="C582" t="s">
+        <v>986</v>
+      </c>
+      <c r="D582" s="10" t="s">
         <v>984</v>
       </c>
-      <c r="D582" s="10" t="s">
-        <v>985</v>
-      </c>
-    </row>
-    <row r="590" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A590" s="2" t="s">
+    </row>
+    <row r="583" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A583" s="2" t="s">
         <v>956</v>
       </c>
-      <c r="D590" s="10" t="s">
+      <c r="B583" t="s">
+        <v>140</v>
+      </c>
+      <c r="D583" s="10" t="s">
         <v>955</v>
       </c>
     </row>
-    <row r="591" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A591" s="2" t="s">
+    <row r="584" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A584" s="2" t="s">
         <v>958</v>
       </c>
-      <c r="D591" s="10" t="s">
+      <c r="B584" t="s">
+        <v>140</v>
+      </c>
+      <c r="D584" s="10" t="s">
         <v>957</v>
+      </c>
+    </row>
+    <row r="585" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A585" s="30" t="s">
+        <v>987</v>
+      </c>
+      <c r="B585" t="s">
+        <v>140</v>
+      </c>
+      <c r="D585" s="10" t="s">
+        <v>988</v>
+      </c>
+    </row>
+    <row r="586" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A586" s="2" t="s">
+        <v>989</v>
+      </c>
+      <c r="B586" t="s">
+        <v>140</v>
+      </c>
+      <c r="D586" s="10" t="s">
+        <v>990</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add PPT workflow and sync-hook refactor updates
</commit_message>
<xml_diff>
--- a/inst/resources/protocol_schema_iphra.xlsx
+++ b/inst/resources/protocol_schema_iphra.xlsx
@@ -5713,7 +5713,7 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C341" s="2" t="inlineStr">
@@ -5735,7 +5735,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C342" s="2" t="inlineStr">
@@ -5757,7 +5757,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C343" s="2" t="inlineStr">
@@ -5779,7 +5779,7 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C344" s="2" t="inlineStr">
@@ -5801,7 +5801,7 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C345" s="2" t="inlineStr">
@@ -5823,7 +5823,7 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C346" s="2" t="inlineStr">
@@ -5845,7 +5845,7 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C347" s="2" t="inlineStr">
@@ -5867,7 +5867,7 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C348" s="2" t="inlineStr">
@@ -5889,7 +5889,7 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C349" s="2" t="inlineStr">
@@ -5911,7 +5911,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C350" s="2" t="inlineStr">
@@ -5933,7 +5933,7 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -5955,7 +5955,7 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C352" s="2" t="inlineStr">
@@ -5977,7 +5977,7 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C353" s="2" t="inlineStr">
@@ -5999,7 +5999,7 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C354" s="2" t="inlineStr">
@@ -6021,7 +6021,7 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
@@ -6043,7 +6043,7 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C356" s="2" t="inlineStr">
@@ -6065,7 +6065,7 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C357" s="2" t="inlineStr">
@@ -6105,7 +6105,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C359" s="2" t="inlineStr">
@@ -6145,7 +6145,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C361" s="2" t="inlineStr">
@@ -6185,7 +6185,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C363" s="2" t="inlineStr">
@@ -6225,7 +6225,7 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C365" s="2" t="inlineStr">
@@ -6265,7 +6265,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C367" s="2" t="inlineStr">
@@ -6305,7 +6305,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C369" s="2" t="inlineStr">
@@ -6345,7 +6345,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C371" s="2" t="inlineStr">
@@ -6385,7 +6385,7 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C373" s="2" t="inlineStr">
@@ -6425,7 +6425,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C375" s="2" t="inlineStr">
@@ -6465,7 +6465,7 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C377" s="2" t="inlineStr">
@@ -6505,7 +6505,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C379" s="2" t="inlineStr">
@@ -6545,7 +6545,7 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C381" s="2" t="inlineStr">
@@ -6585,7 +6585,7 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C383" s="2" t="inlineStr">
@@ -6625,7 +6625,7 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C385" s="2" t="inlineStr">
@@ -6665,7 +6665,7 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C387" s="2" t="inlineStr">
@@ -6687,7 +6687,7 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C388" s="2" t="inlineStr">
@@ -6709,7 +6709,7 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C389" s="2" t="inlineStr">
@@ -6731,7 +6731,7 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C390" s="2" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C391" s="2" t="inlineStr">
@@ -6775,7 +6775,7 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C392" s="2" t="inlineStr">
@@ -6797,7 +6797,7 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C393" s="2" t="inlineStr">
@@ -6819,7 +6819,7 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C394" s="2" t="inlineStr">
@@ -6841,7 +6841,7 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C395" s="2" t="inlineStr">
@@ -6863,7 +6863,7 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C396" s="2" t="inlineStr">
@@ -6885,7 +6885,7 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C397" s="2" t="inlineStr">
@@ -6907,7 +6907,7 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C398" s="2" t="inlineStr">
@@ -7703,7 +7703,7 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C439" s="2" t="inlineStr">
@@ -7725,7 +7725,7 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C440" s="2" t="inlineStr">
@@ -7747,7 +7747,7 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C441" s="2" t="inlineStr">
@@ -7769,7 +7769,7 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C442" s="2" t="inlineStr">
@@ -7791,7 +7791,7 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C443" s="2" t="inlineStr">
@@ -7813,7 +7813,7 @@
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C444" s="2" t="inlineStr">
@@ -7835,7 +7835,7 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>conditional_replace</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="C445" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Address latest PR feedback on orchestration and survey sync
</commit_message>
<xml_diff>
--- a/inst/resources/protocol_schema_iphra.xlsx
+++ b/inst/resources/protocol_schema_iphra.xlsx
@@ -6934,7 +6934,7 @@
       </c>
       <c r="E399" t="inlineStr">
         <is>
-          <t>phr_doc_add_primary_data_sources_table</t>
+          <t>table_primary_data_sources</t>
         </is>
       </c>
     </row>
@@ -7638,11 +7638,7 @@
           <t>image</t>
         </is>
       </c>
-      <c r="E435" t="inlineStr">
-        <is>
-          <t>phr_doc_add_framework_image</t>
-        </is>
-      </c>
+      <c r="E435" t="inlineStr"/>
     </row>
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
@@ -7674,7 +7670,7 @@
       </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t>phr_doc_add_secondary_data_sources_table</t>
+          <t>table_secondary_data_sources</t>
         </is>
       </c>
     </row>
@@ -8152,7 +8148,7 @@
       </c>
       <c r="E464" t="inlineStr">
         <is>
-          <t>phr_doc_add_sample_size_gen_table</t>
+          <t>table_sample_size_general</t>
         </is>
       </c>
     </row>
@@ -8174,7 +8170,7 @@
       </c>
       <c r="E465" t="inlineStr">
         <is>
-          <t>phr_doc_add_sample_size_ind_table</t>
+          <t>table_sample_size_individual</t>
         </is>
       </c>
     </row>
@@ -8196,7 +8192,7 @@
       </c>
       <c r="E466" t="inlineStr">
         <is>
-          <t>phr_doc_add_sample_size_mort_table</t>
+          <t>table_sample_size_mortality</t>
         </is>
       </c>
     </row>

</xml_diff>